<commit_message>
Decide γ denominator: total_customers(g) = live geography customer count (PLC-012, A.10)
- Baseline v2.5 (amended 7 Oct 2026): version row, §4 term, PLC-012, DAT-002 note, Appendix A.10; γ = 1 when count is zero
- Close GAP-γ across reference docs, design docs, mockup plan, user guides, T15 diagram
- Mockup builders: remove Constant/Manual total_customers modes, live SUMIFS by geography, zero rule; workbooks regenerated
- Grounding skill/linter: total_customers now requires PLC-012/A.10 citation and errors on stale spec-gap wording
</commit_message>
<xml_diff>
--- a/Mockups/acrme_region_selection_whatif_4region.xlsx
+++ b/Mockups/acrme_region_selection_whatif_4region.xlsx
@@ -145,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -210,6 +210,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1088,7 +1091,7 @@
     <row r="23">
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>4. Policy — the five weights (sum=1.0), total_customers mode, DR bootstrap / target, min headroom floors.</t>
+          <t>4. Policy — the five weights (sum=1.0), total_customers source (live, PLC-012), DR bootstrap / target, min headroom floors.</t>
         </is>
       </c>
     </row>
@@ -1204,9 +1207,9 @@
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="6" t="inlineStr">
-        <is>
-          <t>• total_customers is undefined in baseline v2.4 — mode selector on Policy (Live/Constant/Manual). γ values illustrative.</t>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>• total_customers(g) = live count of customers in the geography (PLC-012, A.10); γ = 1 when it is zero. Cust Count values are illustrative.</t>
         </is>
       </c>
     </row>
@@ -1265,12 +1268,12 @@
         <f>Setup!B9</f>
         <v/>
       </c>
-      <c r="E3" s="30" t="inlineStr">
+      <c r="E3" s="31" t="inlineStr">
         <is>
           <t>DR SIZING (max-not-sum, A.6 / DR-017)</t>
         </is>
       </c>
-      <c r="H3" s="33" t="inlineStr">
+      <c r="H3" s="34" t="inlineStr">
         <is>
           <t>RANKED CANDIDATE REGIONS  (Rank 1 = highest PS; blank = not a candidate for this mode)</t>
         </is>
@@ -1394,7 +1397,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(1,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J6" s="31">
+      <c r="J6" s="32">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(1,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1406,7 +1409,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(1,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M6" s="31">
+      <c r="M6" s="32">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(1,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1418,7 +1421,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(1,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P6" s="31">
+      <c r="P6" s="32">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(1,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1441,7 +1444,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(2,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J7" s="31">
+      <c r="J7" s="32">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(2,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1453,7 +1456,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(2,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M7" s="31">
+      <c r="M7" s="32">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(2,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1465,7 +1468,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(2,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P7" s="31">
+      <c r="P7" s="32">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(2,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1491,7 +1494,7 @@
           <t>DR Requirement (max-not-sum)</t>
         </is>
       </c>
-      <c r="F8" s="34">
+      <c r="F8" s="35">
         <f>F6*F7</f>
         <v/>
       </c>
@@ -1503,7 +1506,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(3,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J8" s="31">
+      <c r="J8" s="32">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(3,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1515,7 +1518,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(3,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M8" s="31">
+      <c r="M8" s="32">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(3,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1527,7 +1530,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(3,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P8" s="31">
+      <c r="P8" s="32">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(3,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1542,7 +1545,7 @@
         <f>Scoring_Prod!U3</f>
         <v/>
       </c>
-      <c r="C9" s="31">
+      <c r="C9" s="32">
         <f>Scoring_Prod!U4</f>
         <v/>
       </c>
@@ -1563,7 +1566,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(4,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J9" s="31">
+      <c r="J9" s="32">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(4,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1575,7 +1578,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(4,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M9" s="31">
+      <c r="M9" s="32">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(4,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1587,7 +1590,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(4,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P9" s="31">
+      <c r="P9" s="32">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(4,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1602,7 +1605,7 @@
         <f>Scoring_CVAL!U2</f>
         <v/>
       </c>
-      <c r="C10" s="31">
+      <c r="C10" s="32">
         <f>Scoring_CVAL!U3</f>
         <v/>
       </c>
@@ -1623,7 +1626,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(5,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J10" s="31">
+      <c r="J10" s="32">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(5,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1635,7 +1638,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(5,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M10" s="31">
+      <c r="M10" s="32">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(5,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1647,7 +1650,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(5,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P10" s="31">
+      <c r="P10" s="32">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(5,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1662,11 +1665,11 @@
         <f>Scoring_DR!U2</f>
         <v/>
       </c>
-      <c r="C11" s="31">
+      <c r="C11" s="32">
         <f>Scoring_DR!U3</f>
         <v/>
       </c>
-      <c r="E11" s="35" t="inlineStr">
+      <c r="E11" s="36" t="inlineStr">
         <is>
           <t>Note: illustrative — sources = regions in DR scope geography.</t>
         </is>
@@ -1679,7 +1682,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(6,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J11" s="31">
+      <c r="J11" s="32">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(6,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1691,7 +1694,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(6,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M11" s="31">
+      <c r="M11" s="32">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(6,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1703,7 +1706,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(6,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P11" s="31">
+      <c r="P11" s="32">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(6,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1717,7 +1720,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(7,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J12" s="31">
+      <c r="J12" s="32">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(7,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1729,7 +1732,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(7,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M12" s="31">
+      <c r="M12" s="32">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(7,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1741,7 +1744,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(7,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P12" s="31">
+      <c r="P12" s="32">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(7,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1752,7 +1755,7 @@
           <t>Readiness State</t>
         </is>
       </c>
-      <c r="B13" s="34">
+      <c r="B13" s="35">
         <f>IF(B9="NONE ELIGIBLE","QUOTA_DEFICIT / NEEDS EXPLICIT REGION (Prod)",IF(B10="NONE ELIGIBLE","CAPACITY_UNAVAILABLE (CVAL)",IF(B11="NONE ELIGIBLE","READY_WITH_RISK (no DR region)","READY")))</f>
         <v/>
       </c>
@@ -1764,7 +1767,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(8,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J13" s="31">
+      <c r="J13" s="32">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(8,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1776,7 +1779,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(8,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M13" s="31">
+      <c r="M13" s="32">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(8,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1788,7 +1791,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(8,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P13" s="31">
+      <c r="P13" s="32">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(8,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1802,7 +1805,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(9,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J14" s="31">
+      <c r="J14" s="32">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(9,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1814,7 +1817,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(9,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M14" s="31">
+      <c r="M14" s="32">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(9,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1826,7 +1829,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(9,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P14" s="31">
+      <c r="P14" s="32">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(9,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1849,7 +1852,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(10,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J15" s="31">
+      <c r="J15" s="32">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(10,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1861,7 +1864,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(10,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M15" s="31">
+      <c r="M15" s="32">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(10,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1873,7 +1876,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(10,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P15" s="31">
+      <c r="P15" s="32">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(10,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1887,7 +1890,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(11,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J16" s="31">
+      <c r="J16" s="32">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(11,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1899,7 +1902,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(11,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M16" s="31">
+      <c r="M16" s="32">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(11,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1911,7 +1914,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(11,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P16" s="31">
+      <c r="P16" s="32">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(11,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1925,7 +1928,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(12,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J17" s="31">
+      <c r="J17" s="32">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(12,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1937,7 +1940,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(12,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M17" s="31">
+      <c r="M17" s="32">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(12,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1949,7 +1952,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(12,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P17" s="31">
+      <c r="P17" s="32">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(12,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1963,7 +1966,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(13,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J18" s="31">
+      <c r="J18" s="32">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(13,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1975,7 +1978,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(13,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M18" s="31">
+      <c r="M18" s="32">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(13,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1987,7 +1990,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(13,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P18" s="31">
+      <c r="P18" s="32">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(13,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -2001,7 +2004,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(14,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J19" s="31">
+      <c r="J19" s="32">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(14,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -2013,7 +2016,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(14,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M19" s="31">
+      <c r="M19" s="32">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(14,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -2025,7 +2028,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(14,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P19" s="31">
+      <c r="P19" s="32">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(14,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -3114,7 +3117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3206,49 +3209,28 @@
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>total_customers mode (1=Live 2=Constant 3=Manual)</t>
-        </is>
-      </c>
-      <c r="B10" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="23" t="inlineStr">
-        <is>
-          <t>Geography</t>
-        </is>
-      </c>
-      <c r="E10" s="23" t="inlineStr">
-        <is>
-          <t>Constant</t>
+          <t>total_customers source</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>Live geography count (PLC-012)</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>total_customers(g) = customers in geography g with any environment provisioned or being deployed (baseline v2.5 amended, PLC-012 / A.10). Live, not configurable. Workbook stand-in: sum of Cust Count over the geography's regions.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>Manual total_customers</t>
-        </is>
-      </c>
-      <c r="B11" s="24" t="n">
-        <v>300</v>
-      </c>
-      <c r="D11" s="21" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="E11" s="21" t="n">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="D12" s="21" t="inlineStr">
-        <is>
-          <t>EU</t>
-        </is>
-      </c>
-      <c r="E12" s="21" t="n">
-        <v>90</v>
+          <t>γ when total_customers = 0</t>
+        </is>
+      </c>
+      <c r="B11" s="21" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -3260,14 +3242,6 @@
       <c r="B13" s="24" t="n">
         <v>40</v>
       </c>
-      <c r="D13" s="21" t="inlineStr">
-        <is>
-          <t>Australia</t>
-        </is>
-      </c>
-      <c r="E13" s="21" t="n">
-        <v>40</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
@@ -3278,14 +3252,6 @@
       <c r="B14" s="24" t="n">
         <v>0.8</v>
       </c>
-      <c r="D14" s="21" t="inlineStr">
-        <is>
-          <t>Asia Pacific</t>
-        </is>
-      </c>
-      <c r="E14" s="21" t="n">
-        <v>50</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
@@ -3296,14 +3262,6 @@
       <c r="B15" s="24" t="n">
         <v>20</v>
       </c>
-      <c r="D15" s="21" t="inlineStr">
-        <is>
-          <t>Middle East</t>
-        </is>
-      </c>
-      <c r="E15" s="21" t="n">
-        <v>10</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
@@ -3326,6 +3284,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="D10:H11"/>
+  </mergeCells>
   <conditionalFormatting sqref="B8">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"VALID"</formula>
@@ -3521,42 +3482,42 @@
       <c r="E4" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F4" s="27" t="n">
+      <c r="F4" s="28" t="n">
         <v>42492</v>
       </c>
-      <c r="G4" s="27" t="n">
+      <c r="G4" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="H4" s="28">
+      <c r="H4" s="29">
         <f>F4-G4</f>
         <v/>
       </c>
-      <c r="I4" s="27" t="n">
+      <c r="I4" s="28" t="n">
         <v>63738</v>
       </c>
-      <c r="J4" s="27" t="n">
+      <c r="J4" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="K4" s="28">
+      <c r="K4" s="29">
         <f>I4-J4</f>
         <v/>
       </c>
-      <c r="L4" s="27" t="n">
+      <c r="L4" s="28" t="n">
         <v>94710</v>
       </c>
-      <c r="M4" s="27" t="n">
+      <c r="M4" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="N4" s="27" t="n">
+      <c r="N4" s="28" t="n">
         <v>94708</v>
       </c>
-      <c r="O4" s="27" t="n">
+      <c r="O4" s="28" t="n">
         <v>142064</v>
       </c>
-      <c r="P4" s="27" t="n">
+      <c r="P4" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="Q4" s="28">
+      <c r="Q4" s="29">
         <f>O4-P4</f>
         <v/>
       </c>
@@ -3572,7 +3533,7 @@
       <c r="U4" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="V4" s="28" t="inlineStr">
+      <c r="V4" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -3602,42 +3563,42 @@
       <c r="E5" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F5" s="27" t="n">
+      <c r="F5" s="28" t="n">
         <v>42492</v>
       </c>
-      <c r="G5" s="27" t="n">
+      <c r="G5" s="28" t="n">
         <v>12292</v>
       </c>
-      <c r="H5" s="28">
+      <c r="H5" s="29">
         <f>F5-G5</f>
         <v/>
       </c>
-      <c r="I5" s="27" t="n">
+      <c r="I5" s="28" t="n">
         <v>63738</v>
       </c>
-      <c r="J5" s="27" t="n">
+      <c r="J5" s="28" t="n">
         <v>12292</v>
       </c>
-      <c r="K5" s="28">
+      <c r="K5" s="29">
         <f>I5-J5</f>
         <v/>
       </c>
-      <c r="L5" s="27" t="n">
+      <c r="L5" s="28" t="n">
         <v>94710</v>
       </c>
-      <c r="M5" s="27" t="n">
+      <c r="M5" s="28" t="n">
         <v>27398</v>
       </c>
-      <c r="N5" s="27" t="n">
+      <c r="N5" s="28" t="n">
         <v>67312</v>
       </c>
-      <c r="O5" s="27" t="n">
+      <c r="O5" s="28" t="n">
         <v>142064</v>
       </c>
-      <c r="P5" s="27" t="n">
+      <c r="P5" s="28" t="n">
         <v>27398</v>
       </c>
-      <c r="Q5" s="28">
+      <c r="Q5" s="29">
         <f>O5-P5</f>
         <v/>
       </c>
@@ -3653,7 +3614,7 @@
       <c r="U5" s="24" t="n">
         <v>65</v>
       </c>
-      <c r="V5" s="28" t="inlineStr">
+      <c r="V5" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -3683,42 +3644,42 @@
       <c r="E6" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="27" t="n">
+      <c r="F6" s="28" t="n">
         <v>42492</v>
       </c>
-      <c r="G6" s="27" t="n">
+      <c r="G6" s="28" t="n">
         <v>2326</v>
       </c>
-      <c r="H6" s="28">
+      <c r="H6" s="29">
         <f>F6-G6</f>
         <v/>
       </c>
-      <c r="I6" s="27" t="n">
+      <c r="I6" s="28" t="n">
         <v>63738</v>
       </c>
-      <c r="J6" s="27" t="n">
+      <c r="J6" s="28" t="n">
         <v>2326</v>
       </c>
-      <c r="K6" s="28">
+      <c r="K6" s="29">
         <f>I6-J6</f>
         <v/>
       </c>
-      <c r="L6" s="27" t="n">
+      <c r="L6" s="28" t="n">
         <v>94710</v>
       </c>
-      <c r="M6" s="27" t="n">
+      <c r="M6" s="28" t="n">
         <v>5186</v>
       </c>
-      <c r="N6" s="27" t="n">
+      <c r="N6" s="28" t="n">
         <v>89524</v>
       </c>
-      <c r="O6" s="27" t="n">
+      <c r="O6" s="28" t="n">
         <v>142064</v>
       </c>
-      <c r="P6" s="27" t="n">
+      <c r="P6" s="28" t="n">
         <v>5186</v>
       </c>
-      <c r="Q6" s="28">
+      <c r="Q6" s="29">
         <f>O6-P6</f>
         <v/>
       </c>
@@ -3734,7 +3695,7 @@
       <c r="U6" s="24" t="n">
         <v>10</v>
       </c>
-      <c r="V6" s="28" t="inlineStr">
+      <c r="V6" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -3764,42 +3725,42 @@
       <c r="E7" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="27" t="n">
+      <c r="F7" s="28" t="n">
         <v>154178</v>
       </c>
-      <c r="G7" s="27" t="n">
+      <c r="G7" s="28" t="n">
         <v>142756</v>
       </c>
-      <c r="H7" s="28">
+      <c r="H7" s="29">
         <f>F7-G7</f>
         <v/>
       </c>
-      <c r="I7" s="27" t="n">
+      <c r="I7" s="28" t="n">
         <v>231266</v>
       </c>
-      <c r="J7" s="27" t="n">
+      <c r="J7" s="28" t="n">
         <v>142756</v>
       </c>
-      <c r="K7" s="28">
+      <c r="K7" s="29">
         <f>I7-J7</f>
         <v/>
       </c>
-      <c r="L7" s="27" t="n">
+      <c r="L7" s="28" t="n">
         <v>343646</v>
       </c>
-      <c r="M7" s="27" t="n">
+      <c r="M7" s="28" t="n">
         <v>318190</v>
       </c>
-      <c r="N7" s="27" t="n">
+      <c r="N7" s="28" t="n">
         <v>25456</v>
       </c>
-      <c r="O7" s="27" t="n">
+      <c r="O7" s="28" t="n">
         <v>515468</v>
       </c>
-      <c r="P7" s="27" t="n">
+      <c r="P7" s="28" t="n">
         <v>318190</v>
       </c>
-      <c r="Q7" s="28">
+      <c r="Q7" s="29">
         <f>O7-P7</f>
         <v/>
       </c>
@@ -3815,7 +3776,7 @@
       <c r="U7" s="24" t="n">
         <v>150</v>
       </c>
-      <c r="V7" s="28" t="inlineStr">
+      <c r="V7" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -3845,42 +3806,42 @@
       <c r="E8" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="27" t="n">
+      <c r="F8" s="28" t="n">
         <v>13334</v>
       </c>
-      <c r="G8" s="27" t="n">
+      <c r="G8" s="28" t="n">
         <v>628</v>
       </c>
-      <c r="H8" s="28">
+      <c r="H8" s="29">
         <f>F8-G8</f>
         <v/>
       </c>
-      <c r="I8" s="27" t="n">
+      <c r="I8" s="28" t="n">
         <v>20002</v>
       </c>
-      <c r="J8" s="27" t="n">
+      <c r="J8" s="28" t="n">
         <v>628</v>
       </c>
-      <c r="K8" s="28">
+      <c r="K8" s="29">
         <f>I8-J8</f>
         <v/>
       </c>
-      <c r="L8" s="27" t="n">
+      <c r="L8" s="28" t="n">
         <v>40456</v>
       </c>
-      <c r="M8" s="27" t="n">
+      <c r="M8" s="28" t="n">
         <v>1902</v>
       </c>
-      <c r="N8" s="27" t="n">
+      <c r="N8" s="28" t="n">
         <v>38554</v>
       </c>
-      <c r="O8" s="27" t="n">
+      <c r="O8" s="28" t="n">
         <v>60684</v>
       </c>
-      <c r="P8" s="27" t="n">
+      <c r="P8" s="28" t="n">
         <v>1902</v>
       </c>
-      <c r="Q8" s="28">
+      <c r="Q8" s="29">
         <f>O8-P8</f>
         <v/>
       </c>
@@ -3896,7 +3857,7 @@
       <c r="U8" s="24" t="n">
         <v>11</v>
       </c>
-      <c r="V8" s="28" t="inlineStr">
+      <c r="V8" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -3926,42 +3887,42 @@
       <c r="E9" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F9" s="27" t="n">
+      <c r="F9" s="28" t="n">
         <v>13334</v>
       </c>
-      <c r="G9" s="27" t="n">
+      <c r="G9" s="28" t="n">
         <v>842</v>
       </c>
-      <c r="H9" s="28">
+      <c r="H9" s="29">
         <f>F9-G9</f>
         <v/>
       </c>
-      <c r="I9" s="27" t="n">
+      <c r="I9" s="28" t="n">
         <v>20002</v>
       </c>
-      <c r="J9" s="27" t="n">
+      <c r="J9" s="28" t="n">
         <v>842</v>
       </c>
-      <c r="K9" s="28">
+      <c r="K9" s="29">
         <f>I9-J9</f>
         <v/>
       </c>
-      <c r="L9" s="27" t="n">
+      <c r="L9" s="28" t="n">
         <v>40456</v>
       </c>
-      <c r="M9" s="27" t="n">
+      <c r="M9" s="28" t="n">
         <v>2552</v>
       </c>
-      <c r="N9" s="27" t="n">
+      <c r="N9" s="28" t="n">
         <v>37904</v>
       </c>
-      <c r="O9" s="27" t="n">
+      <c r="O9" s="28" t="n">
         <v>60684</v>
       </c>
-      <c r="P9" s="27" t="n">
+      <c r="P9" s="28" t="n">
         <v>2552</v>
       </c>
-      <c r="Q9" s="28">
+      <c r="Q9" s="29">
         <f>O9-P9</f>
         <v/>
       </c>
@@ -3977,7 +3938,7 @@
       <c r="U9" s="24" t="n">
         <v>13</v>
       </c>
-      <c r="V9" s="28" t="inlineStr">
+      <c r="V9" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -4007,42 +3968,42 @@
       <c r="E10" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="27" t="n">
+      <c r="F10" s="28" t="n">
         <v>13334</v>
       </c>
-      <c r="G10" s="27" t="n">
+      <c r="G10" s="28" t="n">
         <v>3072</v>
       </c>
-      <c r="H10" s="28">
+      <c r="H10" s="29">
         <f>F10-G10</f>
         <v/>
       </c>
-      <c r="I10" s="27" t="n">
+      <c r="I10" s="28" t="n">
         <v>20002</v>
       </c>
-      <c r="J10" s="27" t="n">
+      <c r="J10" s="28" t="n">
         <v>3072</v>
       </c>
-      <c r="K10" s="28">
+      <c r="K10" s="29">
         <f>I10-J10</f>
         <v/>
       </c>
-      <c r="L10" s="27" t="n">
+      <c r="L10" s="28" t="n">
         <v>40456</v>
       </c>
-      <c r="M10" s="27" t="n">
+      <c r="M10" s="28" t="n">
         <v>9322</v>
       </c>
-      <c r="N10" s="27" t="n">
+      <c r="N10" s="28" t="n">
         <v>31134</v>
       </c>
-      <c r="O10" s="27" t="n">
+      <c r="O10" s="28" t="n">
         <v>60684</v>
       </c>
-      <c r="P10" s="27" t="n">
+      <c r="P10" s="28" t="n">
         <v>9322</v>
       </c>
-      <c r="Q10" s="28">
+      <c r="Q10" s="29">
         <f>O10-P10</f>
         <v/>
       </c>
@@ -4058,7 +4019,7 @@
       <c r="U10" s="24" t="n">
         <v>30</v>
       </c>
-      <c r="V10" s="28" t="inlineStr">
+      <c r="V10" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -4088,42 +4049,42 @@
       <c r="E11" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F11" s="27" t="n">
+      <c r="F11" s="28" t="n">
         <v>48434</v>
       </c>
-      <c r="G11" s="27" t="n">
+      <c r="G11" s="28" t="n">
         <v>44846</v>
       </c>
-      <c r="H11" s="28">
+      <c r="H11" s="29">
         <f>F11-G11</f>
         <v/>
       </c>
-      <c r="I11" s="27" t="n">
+      <c r="I11" s="28" t="n">
         <v>72650</v>
       </c>
-      <c r="J11" s="27" t="n">
+      <c r="J11" s="28" t="n">
         <v>44846</v>
       </c>
-      <c r="K11" s="28">
+      <c r="K11" s="29">
         <f>I11-J11</f>
         <v/>
       </c>
-      <c r="L11" s="27" t="n">
+      <c r="L11" s="28" t="n">
         <v>146950</v>
       </c>
-      <c r="M11" s="27" t="n">
+      <c r="M11" s="28" t="n">
         <v>136064</v>
       </c>
-      <c r="N11" s="27" t="n">
+      <c r="N11" s="28" t="n">
         <v>10886</v>
       </c>
-      <c r="O11" s="27" t="n">
+      <c r="O11" s="28" t="n">
         <v>220424</v>
       </c>
-      <c r="P11" s="27" t="n">
+      <c r="P11" s="28" t="n">
         <v>136064</v>
       </c>
-      <c r="Q11" s="28">
+      <c r="Q11" s="29">
         <f>O11-P11</f>
         <v/>
       </c>
@@ -4139,7 +4100,7 @@
       <c r="U11" s="24" t="n">
         <v>69</v>
       </c>
-      <c r="V11" s="28" t="inlineStr">
+      <c r="V11" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -4169,42 +4130,42 @@
       <c r="E12" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="28" t="n">
         <v>9518</v>
       </c>
-      <c r="G12" s="27" t="n">
+      <c r="G12" s="28" t="n">
         <v>8812</v>
       </c>
-      <c r="H12" s="28">
+      <c r="H12" s="29">
         <f>F12-G12</f>
         <v/>
       </c>
-      <c r="I12" s="27" t="n">
+      <c r="I12" s="28" t="n">
         <v>14276</v>
       </c>
-      <c r="J12" s="27" t="n">
+      <c r="J12" s="28" t="n">
         <v>8812</v>
       </c>
-      <c r="K12" s="28">
+      <c r="K12" s="29">
         <f>I12-J12</f>
         <v/>
       </c>
-      <c r="L12" s="27" t="n">
+      <c r="L12" s="28" t="n">
         <v>17958</v>
       </c>
-      <c r="M12" s="27" t="n">
+      <c r="M12" s="28" t="n">
         <v>16628</v>
       </c>
-      <c r="N12" s="27" t="n">
+      <c r="N12" s="28" t="n">
         <v>1330</v>
       </c>
-      <c r="O12" s="27" t="n">
+      <c r="O12" s="28" t="n">
         <v>26936</v>
       </c>
-      <c r="P12" s="27" t="n">
+      <c r="P12" s="28" t="n">
         <v>16628</v>
       </c>
-      <c r="Q12" s="28">
+      <c r="Q12" s="29">
         <f>O12-P12</f>
         <v/>
       </c>
@@ -4220,7 +4181,7 @@
       <c r="U12" s="24" t="n">
         <v>34</v>
       </c>
-      <c r="V12" s="28" t="inlineStr">
+      <c r="V12" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -4250,42 +4211,42 @@
       <c r="E13" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="F13" s="27" t="n">
+      <c r="F13" s="28" t="n">
         <v>5624</v>
       </c>
-      <c r="G13" s="27" t="n">
+      <c r="G13" s="28" t="n">
         <v>1602</v>
       </c>
-      <c r="H13" s="28">
+      <c r="H13" s="29">
         <f>F13-G13</f>
         <v/>
       </c>
-      <c r="I13" s="27" t="n">
+      <c r="I13" s="28" t="n">
         <v>8434</v>
       </c>
-      <c r="J13" s="27" t="n">
+      <c r="J13" s="28" t="n">
         <v>1602</v>
       </c>
-      <c r="K13" s="28">
+      <c r="K13" s="29">
         <f>I13-J13</f>
         <v/>
       </c>
-      <c r="L13" s="27" t="n">
+      <c r="L13" s="28" t="n">
         <v>10610</v>
       </c>
-      <c r="M13" s="27" t="n">
+      <c r="M13" s="28" t="n">
         <v>3020</v>
       </c>
-      <c r="N13" s="27" t="n">
+      <c r="N13" s="28" t="n">
         <v>7590</v>
       </c>
-      <c r="O13" s="27" t="n">
+      <c r="O13" s="28" t="n">
         <v>15914</v>
       </c>
-      <c r="P13" s="27" t="n">
+      <c r="P13" s="28" t="n">
         <v>3020</v>
       </c>
-      <c r="Q13" s="28">
+      <c r="Q13" s="29">
         <f>O13-P13</f>
         <v/>
       </c>
@@ -4301,7 +4262,7 @@
       <c r="U13" s="24" t="n">
         <v>14</v>
       </c>
-      <c r="V13" s="28" t="inlineStr">
+      <c r="V13" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -4331,42 +4292,42 @@
       <c r="E14" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F14" s="27" t="n">
+      <c r="F14" s="28" t="n">
         <v>12504</v>
       </c>
-      <c r="G14" s="27" t="n">
+      <c r="G14" s="28" t="n">
         <v>2956</v>
       </c>
-      <c r="H14" s="28">
+      <c r="H14" s="29">
         <f>F14-G14</f>
         <v/>
       </c>
-      <c r="I14" s="27" t="n">
+      <c r="I14" s="28" t="n">
         <v>18756</v>
       </c>
-      <c r="J14" s="27" t="n">
+      <c r="J14" s="28" t="n">
         <v>2956</v>
       </c>
-      <c r="K14" s="28">
+      <c r="K14" s="29">
         <f>I14-J14</f>
         <v/>
       </c>
-      <c r="L14" s="27" t="n">
+      <c r="L14" s="28" t="n">
         <v>13968</v>
       </c>
-      <c r="M14" s="27" t="n">
+      <c r="M14" s="28" t="n">
         <v>3302</v>
       </c>
-      <c r="N14" s="27" t="n">
+      <c r="N14" s="28" t="n">
         <v>10666</v>
       </c>
-      <c r="O14" s="27" t="n">
+      <c r="O14" s="28" t="n">
         <v>20952</v>
       </c>
-      <c r="P14" s="27" t="n">
+      <c r="P14" s="28" t="n">
         <v>3302</v>
       </c>
-      <c r="Q14" s="28">
+      <c r="Q14" s="29">
         <f>O14-P14</f>
         <v/>
       </c>
@@ -4382,7 +4343,7 @@
       <c r="U14" s="24" t="n">
         <v>21</v>
       </c>
-      <c r="V14" s="28" t="inlineStr">
+      <c r="V14" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -4412,42 +4373,42 @@
       <c r="E15" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F15" s="27" t="n">
+      <c r="F15" s="28" t="n">
         <v>21816</v>
       </c>
-      <c r="G15" s="27" t="n">
+      <c r="G15" s="28" t="n">
         <v>20200</v>
       </c>
-      <c r="H15" s="28">
+      <c r="H15" s="29">
         <f>F15-G15</f>
         <v/>
       </c>
-      <c r="I15" s="27" t="n">
+      <c r="I15" s="28" t="n">
         <v>32722</v>
       </c>
-      <c r="J15" s="27" t="n">
+      <c r="J15" s="28" t="n">
         <v>20200</v>
       </c>
-      <c r="K15" s="28">
+      <c r="K15" s="29">
         <f>I15-J15</f>
         <v/>
       </c>
-      <c r="L15" s="27" t="n">
+      <c r="L15" s="28" t="n">
         <v>24370</v>
       </c>
-      <c r="M15" s="27" t="n">
+      <c r="M15" s="28" t="n">
         <v>22566</v>
       </c>
-      <c r="N15" s="27" t="n">
+      <c r="N15" s="28" t="n">
         <v>1804</v>
       </c>
-      <c r="O15" s="27" t="n">
+      <c r="O15" s="28" t="n">
         <v>36556</v>
       </c>
-      <c r="P15" s="27" t="n">
+      <c r="P15" s="28" t="n">
         <v>22566</v>
       </c>
-      <c r="Q15" s="28">
+      <c r="Q15" s="29">
         <f>O15-P15</f>
         <v/>
       </c>
@@ -4463,7 +4424,7 @@
       <c r="U15" s="24" t="n">
         <v>43</v>
       </c>
-      <c r="V15" s="28" t="inlineStr">
+      <c r="V15" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -4493,42 +4454,42 @@
       <c r="E16" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="F16" s="29" t="n">
+      <c r="F16" s="30" t="n">
         <v>1296</v>
       </c>
-      <c r="G16" s="29" t="n">
+      <c r="G16" s="30" t="n">
         <v>1200</v>
       </c>
-      <c r="H16" s="28">
+      <c r="H16" s="29">
         <f>F16-G16</f>
         <v/>
       </c>
-      <c r="I16" s="29" t="n">
+      <c r="I16" s="30" t="n">
         <v>1944</v>
       </c>
-      <c r="J16" s="29" t="n">
+      <c r="J16" s="30" t="n">
         <v>1200</v>
       </c>
-      <c r="K16" s="28">
+      <c r="K16" s="29">
         <f>I16-J16</f>
         <v/>
       </c>
-      <c r="L16" s="29" t="n">
+      <c r="L16" s="30" t="n">
         <v>1838</v>
       </c>
-      <c r="M16" s="29" t="n">
+      <c r="M16" s="30" t="n">
         <v>1700</v>
       </c>
-      <c r="N16" s="29" t="n">
+      <c r="N16" s="30" t="n">
         <v>138</v>
       </c>
-      <c r="O16" s="29" t="n">
+      <c r="O16" s="30" t="n">
         <v>2756</v>
       </c>
-      <c r="P16" s="29" t="n">
+      <c r="P16" s="30" t="n">
         <v>1700</v>
       </c>
-      <c r="Q16" s="28">
+      <c r="Q16" s="29">
         <f>O16-P16</f>
         <v/>
       </c>
@@ -4574,42 +4535,42 @@
       <c r="E17" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="F17" s="29" t="n">
+      <c r="F17" s="30" t="n">
         <v>1296</v>
       </c>
-      <c r="G17" s="29" t="n">
+      <c r="G17" s="30" t="n">
         <v>1200</v>
       </c>
-      <c r="H17" s="28">
+      <c r="H17" s="29">
         <f>F17-G17</f>
         <v/>
       </c>
-      <c r="I17" s="29" t="n">
+      <c r="I17" s="30" t="n">
         <v>1944</v>
       </c>
-      <c r="J17" s="29" t="n">
+      <c r="J17" s="30" t="n">
         <v>1200</v>
       </c>
-      <c r="K17" s="28">
+      <c r="K17" s="29">
         <f>I17-J17</f>
         <v/>
       </c>
-      <c r="L17" s="29" t="n">
+      <c r="L17" s="30" t="n">
         <v>1838</v>
       </c>
-      <c r="M17" s="29" t="n">
+      <c r="M17" s="30" t="n">
         <v>1700</v>
       </c>
-      <c r="N17" s="29" t="n">
+      <c r="N17" s="30" t="n">
         <v>138</v>
       </c>
-      <c r="O17" s="29" t="n">
+      <c r="O17" s="30" t="n">
         <v>2756</v>
       </c>
-      <c r="P17" s="29" t="n">
+      <c r="P17" s="30" t="n">
         <v>1700</v>
       </c>
-      <c r="Q17" s="28">
+      <c r="Q17" s="29">
         <f>O17-P17</f>
         <v/>
       </c>
@@ -5496,7 +5457,7 @@
           <t>PS_Prod — Production Placement Score</t>
         </is>
       </c>
-      <c r="T1" s="30" t="inlineStr">
+      <c r="T1" s="31" t="inlineStr">
         <is>
           <t>PROD WINNER</t>
         </is>
@@ -5641,50 +5602,50 @@
         <v/>
       </c>
       <c r="F4" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C4),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C4,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G4" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C4)</f>
+        <v/>
+      </c>
+      <c r="G4" s="32">
         <f>IFERROR(Capacity_Usage!N4/Capacity_Usage!F4,0)</f>
         <v/>
       </c>
-      <c r="H4" s="31">
+      <c r="H4" s="32">
         <f>MIN(MAX(G4,0),1)</f>
         <v/>
       </c>
-      <c r="I4" s="31">
+      <c r="I4" s="32">
         <f>IFERROR(Capacity_Usage!K4/Capacity_Usage!I4,0)</f>
         <v/>
       </c>
-      <c r="J4" s="31">
+      <c r="J4" s="32">
         <f>MIN(MAX(I4,0),1)</f>
         <v/>
       </c>
-      <c r="K4" s="31">
-        <f>IFERROR(1-Capacity_Usage!U4/F4,0)</f>
-        <v/>
-      </c>
-      <c r="L4" s="31">
+      <c r="K4" s="32">
+        <f>IF(F4=0,Policy!$B$11,1-Capacity_Usage!U4/F4)</f>
+        <v/>
+      </c>
+      <c r="L4" s="32">
         <f>MIN(MAX(K4,0),1)</f>
         <v/>
       </c>
-      <c r="M4" s="31">
+      <c r="M4" s="32">
         <f>IFERROR(Capacity_Usage!T4,0)</f>
         <v/>
       </c>
-      <c r="N4" s="31">
+      <c r="N4" s="32">
         <f>MIN(MAX(M4,0),1)</f>
         <v/>
       </c>
-      <c r="O4" s="31">
+      <c r="O4" s="32">
         <f>Capacity_Usage!E4/3</f>
         <v/>
       </c>
-      <c r="P4" s="31">
+      <c r="P4" s="32">
         <f>MIN(MAX(O4,0),1)</f>
         <v/>
       </c>
-      <c r="Q4" s="31">
+      <c r="Q4" s="32">
         <f>Policy!$B$2*H4+Policy!$B$3*J4+Policy!$B$4*L4+Policy!$B$5*N4+Policy!$B$6*P4</f>
         <v/>
       </c>
@@ -5701,7 +5662,7 @@
           <t>Score</t>
         </is>
       </c>
-      <c r="U4" s="32">
+      <c r="U4" s="33">
         <f>IF(Setup!$B$8&lt;&gt;"",INDEX(Q4:Q17,MATCH(Setup!$B$8,A4:A17,0)),IF(MAX(R4:R17)&lt;0,"",MAX(R4:R17)))</f>
         <v/>
       </c>
@@ -5728,50 +5689,50 @@
         <v/>
       </c>
       <c r="F5" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C5),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C5,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G5" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C5)</f>
+        <v/>
+      </c>
+      <c r="G5" s="32">
         <f>IFERROR(Capacity_Usage!N5/Capacity_Usage!F5,0)</f>
         <v/>
       </c>
-      <c r="H5" s="31">
+      <c r="H5" s="32">
         <f>MIN(MAX(G5,0),1)</f>
         <v/>
       </c>
-      <c r="I5" s="31">
+      <c r="I5" s="32">
         <f>IFERROR(Capacity_Usage!K5/Capacity_Usage!I5,0)</f>
         <v/>
       </c>
-      <c r="J5" s="31">
+      <c r="J5" s="32">
         <f>MIN(MAX(I5,0),1)</f>
         <v/>
       </c>
-      <c r="K5" s="31">
-        <f>IFERROR(1-Capacity_Usage!U5/F5,0)</f>
-        <v/>
-      </c>
-      <c r="L5" s="31">
+      <c r="K5" s="32">
+        <f>IF(F5=0,Policy!$B$11,1-Capacity_Usage!U5/F5)</f>
+        <v/>
+      </c>
+      <c r="L5" s="32">
         <f>MIN(MAX(K5,0),1)</f>
         <v/>
       </c>
-      <c r="M5" s="31">
+      <c r="M5" s="32">
         <f>IFERROR(Capacity_Usage!T5,0)</f>
         <v/>
       </c>
-      <c r="N5" s="31">
+      <c r="N5" s="32">
         <f>MIN(MAX(M5,0),1)</f>
         <v/>
       </c>
-      <c r="O5" s="31">
+      <c r="O5" s="32">
         <f>Capacity_Usage!E5/3</f>
         <v/>
       </c>
-      <c r="P5" s="31">
+      <c r="P5" s="32">
         <f>MIN(MAX(O5,0),1)</f>
         <v/>
       </c>
-      <c r="Q5" s="31">
+      <c r="Q5" s="32">
         <f>Policy!$B$2*H5+Policy!$B$3*J5+Policy!$B$4*L5+Policy!$B$5*N5+Policy!$B$6*P5</f>
         <v/>
       </c>
@@ -5806,50 +5767,50 @@
         <v/>
       </c>
       <c r="F6" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C6),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C6,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G6" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C6)</f>
+        <v/>
+      </c>
+      <c r="G6" s="32">
         <f>IFERROR(Capacity_Usage!N6/Capacity_Usage!F6,0)</f>
         <v/>
       </c>
-      <c r="H6" s="31">
+      <c r="H6" s="32">
         <f>MIN(MAX(G6,0),1)</f>
         <v/>
       </c>
-      <c r="I6" s="31">
+      <c r="I6" s="32">
         <f>IFERROR(Capacity_Usage!K6/Capacity_Usage!I6,0)</f>
         <v/>
       </c>
-      <c r="J6" s="31">
+      <c r="J6" s="32">
         <f>MIN(MAX(I6,0),1)</f>
         <v/>
       </c>
-      <c r="K6" s="31">
-        <f>IFERROR(1-Capacity_Usage!U6/F6,0)</f>
-        <v/>
-      </c>
-      <c r="L6" s="31">
+      <c r="K6" s="32">
+        <f>IF(F6=0,Policy!$B$11,1-Capacity_Usage!U6/F6)</f>
+        <v/>
+      </c>
+      <c r="L6" s="32">
         <f>MIN(MAX(K6,0),1)</f>
         <v/>
       </c>
-      <c r="M6" s="31">
+      <c r="M6" s="32">
         <f>IFERROR(Capacity_Usage!T6,0)</f>
         <v/>
       </c>
-      <c r="N6" s="31">
+      <c r="N6" s="32">
         <f>MIN(MAX(M6,0),1)</f>
         <v/>
       </c>
-      <c r="O6" s="31">
+      <c r="O6" s="32">
         <f>Capacity_Usage!E6/3</f>
         <v/>
       </c>
-      <c r="P6" s="31">
+      <c r="P6" s="32">
         <f>MIN(MAX(O6,0),1)</f>
         <v/>
       </c>
-      <c r="Q6" s="31">
+      <c r="Q6" s="32">
         <f>Policy!$B$2*H6+Policy!$B$3*J6+Policy!$B$4*L6+Policy!$B$5*N6+Policy!$B$6*P6</f>
         <v/>
       </c>
@@ -5884,50 +5845,50 @@
         <v/>
       </c>
       <c r="F7" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C7),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C7,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G7" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C7)</f>
+        <v/>
+      </c>
+      <c r="G7" s="32">
         <f>IFERROR(Capacity_Usage!N7/Capacity_Usage!F7,0)</f>
         <v/>
       </c>
-      <c r="H7" s="31">
+      <c r="H7" s="32">
         <f>MIN(MAX(G7,0),1)</f>
         <v/>
       </c>
-      <c r="I7" s="31">
+      <c r="I7" s="32">
         <f>IFERROR(Capacity_Usage!K7/Capacity_Usage!I7,0)</f>
         <v/>
       </c>
-      <c r="J7" s="31">
+      <c r="J7" s="32">
         <f>MIN(MAX(I7,0),1)</f>
         <v/>
       </c>
-      <c r="K7" s="31">
-        <f>IFERROR(1-Capacity_Usage!U7/F7,0)</f>
-        <v/>
-      </c>
-      <c r="L7" s="31">
+      <c r="K7" s="32">
+        <f>IF(F7=0,Policy!$B$11,1-Capacity_Usage!U7/F7)</f>
+        <v/>
+      </c>
+      <c r="L7" s="32">
         <f>MIN(MAX(K7,0),1)</f>
         <v/>
       </c>
-      <c r="M7" s="31">
+      <c r="M7" s="32">
         <f>IFERROR(Capacity_Usage!T7,0)</f>
         <v/>
       </c>
-      <c r="N7" s="31">
+      <c r="N7" s="32">
         <f>MIN(MAX(M7,0),1)</f>
         <v/>
       </c>
-      <c r="O7" s="31">
+      <c r="O7" s="32">
         <f>Capacity_Usage!E7/3</f>
         <v/>
       </c>
-      <c r="P7" s="31">
+      <c r="P7" s="32">
         <f>MIN(MAX(O7,0),1)</f>
         <v/>
       </c>
-      <c r="Q7" s="31">
+      <c r="Q7" s="32">
         <f>Policy!$B$2*H7+Policy!$B$3*J7+Policy!$B$4*L7+Policy!$B$5*N7+Policy!$B$6*P7</f>
         <v/>
       </c>
@@ -5962,50 +5923,50 @@
         <v/>
       </c>
       <c r="F8" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C8),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C8,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G8" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C8)</f>
+        <v/>
+      </c>
+      <c r="G8" s="32">
         <f>IFERROR(Capacity_Usage!N8/Capacity_Usage!F8,0)</f>
         <v/>
       </c>
-      <c r="H8" s="31">
+      <c r="H8" s="32">
         <f>MIN(MAX(G8,0),1)</f>
         <v/>
       </c>
-      <c r="I8" s="31">
+      <c r="I8" s="32">
         <f>IFERROR(Capacity_Usage!K8/Capacity_Usage!I8,0)</f>
         <v/>
       </c>
-      <c r="J8" s="31">
+      <c r="J8" s="32">
         <f>MIN(MAX(I8,0),1)</f>
         <v/>
       </c>
-      <c r="K8" s="31">
-        <f>IFERROR(1-Capacity_Usage!U8/F8,0)</f>
-        <v/>
-      </c>
-      <c r="L8" s="31">
+      <c r="K8" s="32">
+        <f>IF(F8=0,Policy!$B$11,1-Capacity_Usage!U8/F8)</f>
+        <v/>
+      </c>
+      <c r="L8" s="32">
         <f>MIN(MAX(K8,0),1)</f>
         <v/>
       </c>
-      <c r="M8" s="31">
+      <c r="M8" s="32">
         <f>IFERROR(Capacity_Usage!T8,0)</f>
         <v/>
       </c>
-      <c r="N8" s="31">
+      <c r="N8" s="32">
         <f>MIN(MAX(M8,0),1)</f>
         <v/>
       </c>
-      <c r="O8" s="31">
+      <c r="O8" s="32">
         <f>Capacity_Usage!E8/3</f>
         <v/>
       </c>
-      <c r="P8" s="31">
+      <c r="P8" s="32">
         <f>MIN(MAX(O8,0),1)</f>
         <v/>
       </c>
-      <c r="Q8" s="31">
+      <c r="Q8" s="32">
         <f>Policy!$B$2*H8+Policy!$B$3*J8+Policy!$B$4*L8+Policy!$B$5*N8+Policy!$B$6*P8</f>
         <v/>
       </c>
@@ -6040,50 +6001,50 @@
         <v/>
       </c>
       <c r="F9" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C9),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C9,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G9" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C9)</f>
+        <v/>
+      </c>
+      <c r="G9" s="32">
         <f>IFERROR(Capacity_Usage!N9/Capacity_Usage!F9,0)</f>
         <v/>
       </c>
-      <c r="H9" s="31">
+      <c r="H9" s="32">
         <f>MIN(MAX(G9,0),1)</f>
         <v/>
       </c>
-      <c r="I9" s="31">
+      <c r="I9" s="32">
         <f>IFERROR(Capacity_Usage!K9/Capacity_Usage!I9,0)</f>
         <v/>
       </c>
-      <c r="J9" s="31">
+      <c r="J9" s="32">
         <f>MIN(MAX(I9,0),1)</f>
         <v/>
       </c>
-      <c r="K9" s="31">
-        <f>IFERROR(1-Capacity_Usage!U9/F9,0)</f>
-        <v/>
-      </c>
-      <c r="L9" s="31">
+      <c r="K9" s="32">
+        <f>IF(F9=0,Policy!$B$11,1-Capacity_Usage!U9/F9)</f>
+        <v/>
+      </c>
+      <c r="L9" s="32">
         <f>MIN(MAX(K9,0),1)</f>
         <v/>
       </c>
-      <c r="M9" s="31">
+      <c r="M9" s="32">
         <f>IFERROR(Capacity_Usage!T9,0)</f>
         <v/>
       </c>
-      <c r="N9" s="31">
+      <c r="N9" s="32">
         <f>MIN(MAX(M9,0),1)</f>
         <v/>
       </c>
-      <c r="O9" s="31">
+      <c r="O9" s="32">
         <f>Capacity_Usage!E9/3</f>
         <v/>
       </c>
-      <c r="P9" s="31">
+      <c r="P9" s="32">
         <f>MIN(MAX(O9,0),1)</f>
         <v/>
       </c>
-      <c r="Q9" s="31">
+      <c r="Q9" s="32">
         <f>Policy!$B$2*H9+Policy!$B$3*J9+Policy!$B$4*L9+Policy!$B$5*N9+Policy!$B$6*P9</f>
         <v/>
       </c>
@@ -6118,50 +6079,50 @@
         <v/>
       </c>
       <c r="F10" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C10),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C10,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G10" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C10)</f>
+        <v/>
+      </c>
+      <c r="G10" s="32">
         <f>IFERROR(Capacity_Usage!N10/Capacity_Usage!F10,0)</f>
         <v/>
       </c>
-      <c r="H10" s="31">
+      <c r="H10" s="32">
         <f>MIN(MAX(G10,0),1)</f>
         <v/>
       </c>
-      <c r="I10" s="31">
+      <c r="I10" s="32">
         <f>IFERROR(Capacity_Usage!K10/Capacity_Usage!I10,0)</f>
         <v/>
       </c>
-      <c r="J10" s="31">
+      <c r="J10" s="32">
         <f>MIN(MAX(I10,0),1)</f>
         <v/>
       </c>
-      <c r="K10" s="31">
-        <f>IFERROR(1-Capacity_Usage!U10/F10,0)</f>
-        <v/>
-      </c>
-      <c r="L10" s="31">
+      <c r="K10" s="32">
+        <f>IF(F10=0,Policy!$B$11,1-Capacity_Usage!U10/F10)</f>
+        <v/>
+      </c>
+      <c r="L10" s="32">
         <f>MIN(MAX(K10,0),1)</f>
         <v/>
       </c>
-      <c r="M10" s="31">
+      <c r="M10" s="32">
         <f>IFERROR(Capacity_Usage!T10,0)</f>
         <v/>
       </c>
-      <c r="N10" s="31">
+      <c r="N10" s="32">
         <f>MIN(MAX(M10,0),1)</f>
         <v/>
       </c>
-      <c r="O10" s="31">
+      <c r="O10" s="32">
         <f>Capacity_Usage!E10/3</f>
         <v/>
       </c>
-      <c r="P10" s="31">
+      <c r="P10" s="32">
         <f>MIN(MAX(O10,0),1)</f>
         <v/>
       </c>
-      <c r="Q10" s="31">
+      <c r="Q10" s="32">
         <f>Policy!$B$2*H10+Policy!$B$3*J10+Policy!$B$4*L10+Policy!$B$5*N10+Policy!$B$6*P10</f>
         <v/>
       </c>
@@ -6196,50 +6157,50 @@
         <v/>
       </c>
       <c r="F11" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C11),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C11,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G11" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C11)</f>
+        <v/>
+      </c>
+      <c r="G11" s="32">
         <f>IFERROR(Capacity_Usage!N11/Capacity_Usage!F11,0)</f>
         <v/>
       </c>
-      <c r="H11" s="31">
+      <c r="H11" s="32">
         <f>MIN(MAX(G11,0),1)</f>
         <v/>
       </c>
-      <c r="I11" s="31">
+      <c r="I11" s="32">
         <f>IFERROR(Capacity_Usage!K11/Capacity_Usage!I11,0)</f>
         <v/>
       </c>
-      <c r="J11" s="31">
+      <c r="J11" s="32">
         <f>MIN(MAX(I11,0),1)</f>
         <v/>
       </c>
-      <c r="K11" s="31">
-        <f>IFERROR(1-Capacity_Usage!U11/F11,0)</f>
-        <v/>
-      </c>
-      <c r="L11" s="31">
+      <c r="K11" s="32">
+        <f>IF(F11=0,Policy!$B$11,1-Capacity_Usage!U11/F11)</f>
+        <v/>
+      </c>
+      <c r="L11" s="32">
         <f>MIN(MAX(K11,0),1)</f>
         <v/>
       </c>
-      <c r="M11" s="31">
+      <c r="M11" s="32">
         <f>IFERROR(Capacity_Usage!T11,0)</f>
         <v/>
       </c>
-      <c r="N11" s="31">
+      <c r="N11" s="32">
         <f>MIN(MAX(M11,0),1)</f>
         <v/>
       </c>
-      <c r="O11" s="31">
+      <c r="O11" s="32">
         <f>Capacity_Usage!E11/3</f>
         <v/>
       </c>
-      <c r="P11" s="31">
+      <c r="P11" s="32">
         <f>MIN(MAX(O11,0),1)</f>
         <v/>
       </c>
-      <c r="Q11" s="31">
+      <c r="Q11" s="32">
         <f>Policy!$B$2*H11+Policy!$B$3*J11+Policy!$B$4*L11+Policy!$B$5*N11+Policy!$B$6*P11</f>
         <v/>
       </c>
@@ -6274,50 +6235,50 @@
         <v/>
       </c>
       <c r="F12" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C12),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C12,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G12" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C12)</f>
+        <v/>
+      </c>
+      <c r="G12" s="32">
         <f>IFERROR(Capacity_Usage!N12/Capacity_Usage!F12,0)</f>
         <v/>
       </c>
-      <c r="H12" s="31">
+      <c r="H12" s="32">
         <f>MIN(MAX(G12,0),1)</f>
         <v/>
       </c>
-      <c r="I12" s="31">
+      <c r="I12" s="32">
         <f>IFERROR(Capacity_Usage!K12/Capacity_Usage!I12,0)</f>
         <v/>
       </c>
-      <c r="J12" s="31">
+      <c r="J12" s="32">
         <f>MIN(MAX(I12,0),1)</f>
         <v/>
       </c>
-      <c r="K12" s="31">
-        <f>IFERROR(1-Capacity_Usage!U12/F12,0)</f>
-        <v/>
-      </c>
-      <c r="L12" s="31">
+      <c r="K12" s="32">
+        <f>IF(F12=0,Policy!$B$11,1-Capacity_Usage!U12/F12)</f>
+        <v/>
+      </c>
+      <c r="L12" s="32">
         <f>MIN(MAX(K12,0),1)</f>
         <v/>
       </c>
-      <c r="M12" s="31">
+      <c r="M12" s="32">
         <f>IFERROR(Capacity_Usage!T12,0)</f>
         <v/>
       </c>
-      <c r="N12" s="31">
+      <c r="N12" s="32">
         <f>MIN(MAX(M12,0),1)</f>
         <v/>
       </c>
-      <c r="O12" s="31">
+      <c r="O12" s="32">
         <f>Capacity_Usage!E12/3</f>
         <v/>
       </c>
-      <c r="P12" s="31">
+      <c r="P12" s="32">
         <f>MIN(MAX(O12,0),1)</f>
         <v/>
       </c>
-      <c r="Q12" s="31">
+      <c r="Q12" s="32">
         <f>Policy!$B$2*H12+Policy!$B$3*J12+Policy!$B$4*L12+Policy!$B$5*N12+Policy!$B$6*P12</f>
         <v/>
       </c>
@@ -6352,50 +6313,50 @@
         <v/>
       </c>
       <c r="F13" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C13),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C13,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G13" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C13)</f>
+        <v/>
+      </c>
+      <c r="G13" s="32">
         <f>IFERROR(Capacity_Usage!N13/Capacity_Usage!F13,0)</f>
         <v/>
       </c>
-      <c r="H13" s="31">
+      <c r="H13" s="32">
         <f>MIN(MAX(G13,0),1)</f>
         <v/>
       </c>
-      <c r="I13" s="31">
+      <c r="I13" s="32">
         <f>IFERROR(Capacity_Usage!K13/Capacity_Usage!I13,0)</f>
         <v/>
       </c>
-      <c r="J13" s="31">
+      <c r="J13" s="32">
         <f>MIN(MAX(I13,0),1)</f>
         <v/>
       </c>
-      <c r="K13" s="31">
-        <f>IFERROR(1-Capacity_Usage!U13/F13,0)</f>
-        <v/>
-      </c>
-      <c r="L13" s="31">
+      <c r="K13" s="32">
+        <f>IF(F13=0,Policy!$B$11,1-Capacity_Usage!U13/F13)</f>
+        <v/>
+      </c>
+      <c r="L13" s="32">
         <f>MIN(MAX(K13,0),1)</f>
         <v/>
       </c>
-      <c r="M13" s="31">
+      <c r="M13" s="32">
         <f>IFERROR(Capacity_Usage!T13,0)</f>
         <v/>
       </c>
-      <c r="N13" s="31">
+      <c r="N13" s="32">
         <f>MIN(MAX(M13,0),1)</f>
         <v/>
       </c>
-      <c r="O13" s="31">
+      <c r="O13" s="32">
         <f>Capacity_Usage!E13/3</f>
         <v/>
       </c>
-      <c r="P13" s="31">
+      <c r="P13" s="32">
         <f>MIN(MAX(O13,0),1)</f>
         <v/>
       </c>
-      <c r="Q13" s="31">
+      <c r="Q13" s="32">
         <f>Policy!$B$2*H13+Policy!$B$3*J13+Policy!$B$4*L13+Policy!$B$5*N13+Policy!$B$6*P13</f>
         <v/>
       </c>
@@ -6430,50 +6391,50 @@
         <v/>
       </c>
       <c r="F14" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C14),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C14,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G14" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C14)</f>
+        <v/>
+      </c>
+      <c r="G14" s="32">
         <f>IFERROR(Capacity_Usage!N14/Capacity_Usage!F14,0)</f>
         <v/>
       </c>
-      <c r="H14" s="31">
+      <c r="H14" s="32">
         <f>MIN(MAX(G14,0),1)</f>
         <v/>
       </c>
-      <c r="I14" s="31">
+      <c r="I14" s="32">
         <f>IFERROR(Capacity_Usage!K14/Capacity_Usage!I14,0)</f>
         <v/>
       </c>
-      <c r="J14" s="31">
+      <c r="J14" s="32">
         <f>MIN(MAX(I14,0),1)</f>
         <v/>
       </c>
-      <c r="K14" s="31">
-        <f>IFERROR(1-Capacity_Usage!U14/F14,0)</f>
-        <v/>
-      </c>
-      <c r="L14" s="31">
+      <c r="K14" s="32">
+        <f>IF(F14=0,Policy!$B$11,1-Capacity_Usage!U14/F14)</f>
+        <v/>
+      </c>
+      <c r="L14" s="32">
         <f>MIN(MAX(K14,0),1)</f>
         <v/>
       </c>
-      <c r="M14" s="31">
+      <c r="M14" s="32">
         <f>IFERROR(Capacity_Usage!T14,0)</f>
         <v/>
       </c>
-      <c r="N14" s="31">
+      <c r="N14" s="32">
         <f>MIN(MAX(M14,0),1)</f>
         <v/>
       </c>
-      <c r="O14" s="31">
+      <c r="O14" s="32">
         <f>Capacity_Usage!E14/3</f>
         <v/>
       </c>
-      <c r="P14" s="31">
+      <c r="P14" s="32">
         <f>MIN(MAX(O14,0),1)</f>
         <v/>
       </c>
-      <c r="Q14" s="31">
+      <c r="Q14" s="32">
         <f>Policy!$B$2*H14+Policy!$B$3*J14+Policy!$B$4*L14+Policy!$B$5*N14+Policy!$B$6*P14</f>
         <v/>
       </c>
@@ -6508,50 +6469,50 @@
         <v/>
       </c>
       <c r="F15" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C15),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C15,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G15" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C15)</f>
+        <v/>
+      </c>
+      <c r="G15" s="32">
         <f>IFERROR(Capacity_Usage!N15/Capacity_Usage!F15,0)</f>
         <v/>
       </c>
-      <c r="H15" s="31">
+      <c r="H15" s="32">
         <f>MIN(MAX(G15,0),1)</f>
         <v/>
       </c>
-      <c r="I15" s="31">
+      <c r="I15" s="32">
         <f>IFERROR(Capacity_Usage!K15/Capacity_Usage!I15,0)</f>
         <v/>
       </c>
-      <c r="J15" s="31">
+      <c r="J15" s="32">
         <f>MIN(MAX(I15,0),1)</f>
         <v/>
       </c>
-      <c r="K15" s="31">
-        <f>IFERROR(1-Capacity_Usage!U15/F15,0)</f>
-        <v/>
-      </c>
-      <c r="L15" s="31">
+      <c r="K15" s="32">
+        <f>IF(F15=0,Policy!$B$11,1-Capacity_Usage!U15/F15)</f>
+        <v/>
+      </c>
+      <c r="L15" s="32">
         <f>MIN(MAX(K15,0),1)</f>
         <v/>
       </c>
-      <c r="M15" s="31">
+      <c r="M15" s="32">
         <f>IFERROR(Capacity_Usage!T15,0)</f>
         <v/>
       </c>
-      <c r="N15" s="31">
+      <c r="N15" s="32">
         <f>MIN(MAX(M15,0),1)</f>
         <v/>
       </c>
-      <c r="O15" s="31">
+      <c r="O15" s="32">
         <f>Capacity_Usage!E15/3</f>
         <v/>
       </c>
-      <c r="P15" s="31">
+      <c r="P15" s="32">
         <f>MIN(MAX(O15,0),1)</f>
         <v/>
       </c>
-      <c r="Q15" s="31">
+      <c r="Q15" s="32">
         <f>Policy!$B$2*H15+Policy!$B$3*J15+Policy!$B$4*L15+Policy!$B$5*N15+Policy!$B$6*P15</f>
         <v/>
       </c>
@@ -6586,50 +6547,50 @@
         <v/>
       </c>
       <c r="F16" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C16),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C16,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G16" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C16)</f>
+        <v/>
+      </c>
+      <c r="G16" s="32">
         <f>IFERROR(Capacity_Usage!N16/Capacity_Usage!F16,0)</f>
         <v/>
       </c>
-      <c r="H16" s="31">
+      <c r="H16" s="32">
         <f>MIN(MAX(G16,0),1)</f>
         <v/>
       </c>
-      <c r="I16" s="31">
+      <c r="I16" s="32">
         <f>IFERROR(Capacity_Usage!K16/Capacity_Usage!I16,0)</f>
         <v/>
       </c>
-      <c r="J16" s="31">
+      <c r="J16" s="32">
         <f>MIN(MAX(I16,0),1)</f>
         <v/>
       </c>
-      <c r="K16" s="31">
-        <f>IFERROR(1-Capacity_Usage!U16/F16,0)</f>
-        <v/>
-      </c>
-      <c r="L16" s="31">
+      <c r="K16" s="32">
+        <f>IF(F16=0,Policy!$B$11,1-Capacity_Usage!U16/F16)</f>
+        <v/>
+      </c>
+      <c r="L16" s="32">
         <f>MIN(MAX(K16,0),1)</f>
         <v/>
       </c>
-      <c r="M16" s="31">
+      <c r="M16" s="32">
         <f>IFERROR(Capacity_Usage!T16,0)</f>
         <v/>
       </c>
-      <c r="N16" s="31">
+      <c r="N16" s="32">
         <f>MIN(MAX(M16,0),1)</f>
         <v/>
       </c>
-      <c r="O16" s="31">
+      <c r="O16" s="32">
         <f>Capacity_Usage!E16/3</f>
         <v/>
       </c>
-      <c r="P16" s="31">
+      <c r="P16" s="32">
         <f>MIN(MAX(O16,0),1)</f>
         <v/>
       </c>
-      <c r="Q16" s="31">
+      <c r="Q16" s="32">
         <f>Policy!$B$2*H16+Policy!$B$3*J16+Policy!$B$4*L16+Policy!$B$5*N16+Policy!$B$6*P16</f>
         <v/>
       </c>
@@ -6664,50 +6625,50 @@
         <v/>
       </c>
       <c r="F17" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C17),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C17,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G17" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C17)</f>
+        <v/>
+      </c>
+      <c r="G17" s="32">
         <f>IFERROR(Capacity_Usage!N17/Capacity_Usage!F17,0)</f>
         <v/>
       </c>
-      <c r="H17" s="31">
+      <c r="H17" s="32">
         <f>MIN(MAX(G17,0),1)</f>
         <v/>
       </c>
-      <c r="I17" s="31">
+      <c r="I17" s="32">
         <f>IFERROR(Capacity_Usage!K17/Capacity_Usage!I17,0)</f>
         <v/>
       </c>
-      <c r="J17" s="31">
+      <c r="J17" s="32">
         <f>MIN(MAX(I17,0),1)</f>
         <v/>
       </c>
-      <c r="K17" s="31">
-        <f>IFERROR(1-Capacity_Usage!U17/F17,0)</f>
-        <v/>
-      </c>
-      <c r="L17" s="31">
+      <c r="K17" s="32">
+        <f>IF(F17=0,Policy!$B$11,1-Capacity_Usage!U17/F17)</f>
+        <v/>
+      </c>
+      <c r="L17" s="32">
         <f>MIN(MAX(K17,0),1)</f>
         <v/>
       </c>
-      <c r="M17" s="31">
+      <c r="M17" s="32">
         <f>IFERROR(Capacity_Usage!T17,0)</f>
         <v/>
       </c>
-      <c r="N17" s="31">
+      <c r="N17" s="32">
         <f>MIN(MAX(M17,0),1)</f>
         <v/>
       </c>
-      <c r="O17" s="31">
+      <c r="O17" s="32">
         <f>Capacity_Usage!E17/3</f>
         <v/>
       </c>
-      <c r="P17" s="31">
+      <c r="P17" s="32">
         <f>MIN(MAX(O17,0),1)</f>
         <v/>
       </c>
-      <c r="Q17" s="31">
+      <c r="Q17" s="32">
         <f>Policy!$B$2*H17+Policy!$B$3*J17+Policy!$B$4*L17+Policy!$B$5*N17+Policy!$B$6*P17</f>
         <v/>
       </c>
@@ -6764,7 +6725,7 @@
           <t>PS_NonProd — CVAL Placement Score  (δ duplicates α — known design gap)</t>
         </is>
       </c>
-      <c r="T1" s="30" t="inlineStr">
+      <c r="T1" s="31" t="inlineStr">
         <is>
           <t>CVAL WINNER</t>
         </is>
@@ -6882,7 +6843,7 @@
           <t>Score</t>
         </is>
       </c>
-      <c r="U3" s="32">
+      <c r="U3" s="33">
         <f>IF(Setup!$B$3="Middle East",Scoring_Prod!$U$4,IF(MAX(R4:R17)&lt;0,"",MAX(R4:R17)))</f>
         <v/>
       </c>
@@ -6909,50 +6870,50 @@
         <v/>
       </c>
       <c r="F4" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C4),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C4,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G4" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C4)</f>
+        <v/>
+      </c>
+      <c r="G4" s="32">
         <f>IFERROR(Capacity_Usage!N4/Capacity_Usage!L4,0)</f>
         <v/>
       </c>
-      <c r="H4" s="31">
+      <c r="H4" s="32">
         <f>MIN(MAX(G4,0),1)</f>
         <v/>
       </c>
-      <c r="I4" s="31">
+      <c r="I4" s="32">
         <f>IFERROR(Capacity_Usage!Q4/Capacity_Usage!O4,0)</f>
         <v/>
       </c>
-      <c r="J4" s="31">
+      <c r="J4" s="32">
         <f>MIN(MAX(I4,0),1)</f>
         <v/>
       </c>
-      <c r="K4" s="31">
-        <f>IFERROR(1-Capacity_Usage!U4/F4,0)</f>
-        <v/>
-      </c>
-      <c r="L4" s="31">
+      <c r="K4" s="32">
+        <f>IF(F4=0,Policy!$B$11,1-Capacity_Usage!U4/F4)</f>
+        <v/>
+      </c>
+      <c r="L4" s="32">
         <f>MIN(MAX(K4,0),1)</f>
         <v/>
       </c>
-      <c r="M4" s="31">
+      <c r="M4" s="32">
         <f>IFERROR(Capacity_Usage!N4/Capacity_Usage!L4,0)</f>
         <v/>
       </c>
-      <c r="N4" s="31">
+      <c r="N4" s="32">
         <f>MIN(MAX(M4,0),1)</f>
         <v/>
       </c>
-      <c r="O4" s="31">
+      <c r="O4" s="32">
         <f>Capacity_Usage!E4/3</f>
         <v/>
       </c>
-      <c r="P4" s="31">
+      <c r="P4" s="32">
         <f>MIN(MAX(O4,0),1)</f>
         <v/>
       </c>
-      <c r="Q4" s="31">
+      <c r="Q4" s="32">
         <f>Policy!$B$2*H4+Policy!$B$3*J4+Policy!$B$4*L4+Policy!$B$5*N4+Policy!$B$6*P4</f>
         <v/>
       </c>
@@ -6987,50 +6948,50 @@
         <v/>
       </c>
       <c r="F5" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C5),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C5,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G5" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C5)</f>
+        <v/>
+      </c>
+      <c r="G5" s="32">
         <f>IFERROR(Capacity_Usage!N5/Capacity_Usage!L5,0)</f>
         <v/>
       </c>
-      <c r="H5" s="31">
+      <c r="H5" s="32">
         <f>MIN(MAX(G5,0),1)</f>
         <v/>
       </c>
-      <c r="I5" s="31">
+      <c r="I5" s="32">
         <f>IFERROR(Capacity_Usage!Q5/Capacity_Usage!O5,0)</f>
         <v/>
       </c>
-      <c r="J5" s="31">
+      <c r="J5" s="32">
         <f>MIN(MAX(I5,0),1)</f>
         <v/>
       </c>
-      <c r="K5" s="31">
-        <f>IFERROR(1-Capacity_Usage!U5/F5,0)</f>
-        <v/>
-      </c>
-      <c r="L5" s="31">
+      <c r="K5" s="32">
+        <f>IF(F5=0,Policy!$B$11,1-Capacity_Usage!U5/F5)</f>
+        <v/>
+      </c>
+      <c r="L5" s="32">
         <f>MIN(MAX(K5,0),1)</f>
         <v/>
       </c>
-      <c r="M5" s="31">
+      <c r="M5" s="32">
         <f>IFERROR(Capacity_Usage!N5/Capacity_Usage!L5,0)</f>
         <v/>
       </c>
-      <c r="N5" s="31">
+      <c r="N5" s="32">
         <f>MIN(MAX(M5,0),1)</f>
         <v/>
       </c>
-      <c r="O5" s="31">
+      <c r="O5" s="32">
         <f>Capacity_Usage!E5/3</f>
         <v/>
       </c>
-      <c r="P5" s="31">
+      <c r="P5" s="32">
         <f>MIN(MAX(O5,0),1)</f>
         <v/>
       </c>
-      <c r="Q5" s="31">
+      <c r="Q5" s="32">
         <f>Policy!$B$2*H5+Policy!$B$3*J5+Policy!$B$4*L5+Policy!$B$5*N5+Policy!$B$6*P5</f>
         <v/>
       </c>
@@ -7065,50 +7026,50 @@
         <v/>
       </c>
       <c r="F6" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C6),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C6,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G6" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C6)</f>
+        <v/>
+      </c>
+      <c r="G6" s="32">
         <f>IFERROR(Capacity_Usage!N6/Capacity_Usage!L6,0)</f>
         <v/>
       </c>
-      <c r="H6" s="31">
+      <c r="H6" s="32">
         <f>MIN(MAX(G6,0),1)</f>
         <v/>
       </c>
-      <c r="I6" s="31">
+      <c r="I6" s="32">
         <f>IFERROR(Capacity_Usage!Q6/Capacity_Usage!O6,0)</f>
         <v/>
       </c>
-      <c r="J6" s="31">
+      <c r="J6" s="32">
         <f>MIN(MAX(I6,0),1)</f>
         <v/>
       </c>
-      <c r="K6" s="31">
-        <f>IFERROR(1-Capacity_Usage!U6/F6,0)</f>
-        <v/>
-      </c>
-      <c r="L6" s="31">
+      <c r="K6" s="32">
+        <f>IF(F6=0,Policy!$B$11,1-Capacity_Usage!U6/F6)</f>
+        <v/>
+      </c>
+      <c r="L6" s="32">
         <f>MIN(MAX(K6,0),1)</f>
         <v/>
       </c>
-      <c r="M6" s="31">
+      <c r="M6" s="32">
         <f>IFERROR(Capacity_Usage!N6/Capacity_Usage!L6,0)</f>
         <v/>
       </c>
-      <c r="N6" s="31">
+      <c r="N6" s="32">
         <f>MIN(MAX(M6,0),1)</f>
         <v/>
       </c>
-      <c r="O6" s="31">
+      <c r="O6" s="32">
         <f>Capacity_Usage!E6/3</f>
         <v/>
       </c>
-      <c r="P6" s="31">
+      <c r="P6" s="32">
         <f>MIN(MAX(O6,0),1)</f>
         <v/>
       </c>
-      <c r="Q6" s="31">
+      <c r="Q6" s="32">
         <f>Policy!$B$2*H6+Policy!$B$3*J6+Policy!$B$4*L6+Policy!$B$5*N6+Policy!$B$6*P6</f>
         <v/>
       </c>
@@ -7143,50 +7104,50 @@
         <v/>
       </c>
       <c r="F7" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C7),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C7,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G7" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C7)</f>
+        <v/>
+      </c>
+      <c r="G7" s="32">
         <f>IFERROR(Capacity_Usage!N7/Capacity_Usage!L7,0)</f>
         <v/>
       </c>
-      <c r="H7" s="31">
+      <c r="H7" s="32">
         <f>MIN(MAX(G7,0),1)</f>
         <v/>
       </c>
-      <c r="I7" s="31">
+      <c r="I7" s="32">
         <f>IFERROR(Capacity_Usage!Q7/Capacity_Usage!O7,0)</f>
         <v/>
       </c>
-      <c r="J7" s="31">
+      <c r="J7" s="32">
         <f>MIN(MAX(I7,0),1)</f>
         <v/>
       </c>
-      <c r="K7" s="31">
-        <f>IFERROR(1-Capacity_Usage!U7/F7,0)</f>
-        <v/>
-      </c>
-      <c r="L7" s="31">
+      <c r="K7" s="32">
+        <f>IF(F7=0,Policy!$B$11,1-Capacity_Usage!U7/F7)</f>
+        <v/>
+      </c>
+      <c r="L7" s="32">
         <f>MIN(MAX(K7,0),1)</f>
         <v/>
       </c>
-      <c r="M7" s="31">
+      <c r="M7" s="32">
         <f>IFERROR(Capacity_Usage!N7/Capacity_Usage!L7,0)</f>
         <v/>
       </c>
-      <c r="N7" s="31">
+      <c r="N7" s="32">
         <f>MIN(MAX(M7,0),1)</f>
         <v/>
       </c>
-      <c r="O7" s="31">
+      <c r="O7" s="32">
         <f>Capacity_Usage!E7/3</f>
         <v/>
       </c>
-      <c r="P7" s="31">
+      <c r="P7" s="32">
         <f>MIN(MAX(O7,0),1)</f>
         <v/>
       </c>
-      <c r="Q7" s="31">
+      <c r="Q7" s="32">
         <f>Policy!$B$2*H7+Policy!$B$3*J7+Policy!$B$4*L7+Policy!$B$5*N7+Policy!$B$6*P7</f>
         <v/>
       </c>
@@ -7221,50 +7182,50 @@
         <v/>
       </c>
       <c r="F8" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C8),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C8,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G8" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C8)</f>
+        <v/>
+      </c>
+      <c r="G8" s="32">
         <f>IFERROR(Capacity_Usage!N8/Capacity_Usage!L8,0)</f>
         <v/>
       </c>
-      <c r="H8" s="31">
+      <c r="H8" s="32">
         <f>MIN(MAX(G8,0),1)</f>
         <v/>
       </c>
-      <c r="I8" s="31">
+      <c r="I8" s="32">
         <f>IFERROR(Capacity_Usage!Q8/Capacity_Usage!O8,0)</f>
         <v/>
       </c>
-      <c r="J8" s="31">
+      <c r="J8" s="32">
         <f>MIN(MAX(I8,0),1)</f>
         <v/>
       </c>
-      <c r="K8" s="31">
-        <f>IFERROR(1-Capacity_Usage!U8/F8,0)</f>
-        <v/>
-      </c>
-      <c r="L8" s="31">
+      <c r="K8" s="32">
+        <f>IF(F8=0,Policy!$B$11,1-Capacity_Usage!U8/F8)</f>
+        <v/>
+      </c>
+      <c r="L8" s="32">
         <f>MIN(MAX(K8,0),1)</f>
         <v/>
       </c>
-      <c r="M8" s="31">
+      <c r="M8" s="32">
         <f>IFERROR(Capacity_Usage!N8/Capacity_Usage!L8,0)</f>
         <v/>
       </c>
-      <c r="N8" s="31">
+      <c r="N8" s="32">
         <f>MIN(MAX(M8,0),1)</f>
         <v/>
       </c>
-      <c r="O8" s="31">
+      <c r="O8" s="32">
         <f>Capacity_Usage!E8/3</f>
         <v/>
       </c>
-      <c r="P8" s="31">
+      <c r="P8" s="32">
         <f>MIN(MAX(O8,0),1)</f>
         <v/>
       </c>
-      <c r="Q8" s="31">
+      <c r="Q8" s="32">
         <f>Policy!$B$2*H8+Policy!$B$3*J8+Policy!$B$4*L8+Policy!$B$5*N8+Policy!$B$6*P8</f>
         <v/>
       </c>
@@ -7299,50 +7260,50 @@
         <v/>
       </c>
       <c r="F9" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C9),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C9,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G9" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C9)</f>
+        <v/>
+      </c>
+      <c r="G9" s="32">
         <f>IFERROR(Capacity_Usage!N9/Capacity_Usage!L9,0)</f>
         <v/>
       </c>
-      <c r="H9" s="31">
+      <c r="H9" s="32">
         <f>MIN(MAX(G9,0),1)</f>
         <v/>
       </c>
-      <c r="I9" s="31">
+      <c r="I9" s="32">
         <f>IFERROR(Capacity_Usage!Q9/Capacity_Usage!O9,0)</f>
         <v/>
       </c>
-      <c r="J9" s="31">
+      <c r="J9" s="32">
         <f>MIN(MAX(I9,0),1)</f>
         <v/>
       </c>
-      <c r="K9" s="31">
-        <f>IFERROR(1-Capacity_Usage!U9/F9,0)</f>
-        <v/>
-      </c>
-      <c r="L9" s="31">
+      <c r="K9" s="32">
+        <f>IF(F9=0,Policy!$B$11,1-Capacity_Usage!U9/F9)</f>
+        <v/>
+      </c>
+      <c r="L9" s="32">
         <f>MIN(MAX(K9,0),1)</f>
         <v/>
       </c>
-      <c r="M9" s="31">
+      <c r="M9" s="32">
         <f>IFERROR(Capacity_Usage!N9/Capacity_Usage!L9,0)</f>
         <v/>
       </c>
-      <c r="N9" s="31">
+      <c r="N9" s="32">
         <f>MIN(MAX(M9,0),1)</f>
         <v/>
       </c>
-      <c r="O9" s="31">
+      <c r="O9" s="32">
         <f>Capacity_Usage!E9/3</f>
         <v/>
       </c>
-      <c r="P9" s="31">
+      <c r="P9" s="32">
         <f>MIN(MAX(O9,0),1)</f>
         <v/>
       </c>
-      <c r="Q9" s="31">
+      <c r="Q9" s="32">
         <f>Policy!$B$2*H9+Policy!$B$3*J9+Policy!$B$4*L9+Policy!$B$5*N9+Policy!$B$6*P9</f>
         <v/>
       </c>
@@ -7377,50 +7338,50 @@
         <v/>
       </c>
       <c r="F10" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C10),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C10,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G10" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C10)</f>
+        <v/>
+      </c>
+      <c r="G10" s="32">
         <f>IFERROR(Capacity_Usage!N10/Capacity_Usage!L10,0)</f>
         <v/>
       </c>
-      <c r="H10" s="31">
+      <c r="H10" s="32">
         <f>MIN(MAX(G10,0),1)</f>
         <v/>
       </c>
-      <c r="I10" s="31">
+      <c r="I10" s="32">
         <f>IFERROR(Capacity_Usage!Q10/Capacity_Usage!O10,0)</f>
         <v/>
       </c>
-      <c r="J10" s="31">
+      <c r="J10" s="32">
         <f>MIN(MAX(I10,0),1)</f>
         <v/>
       </c>
-      <c r="K10" s="31">
-        <f>IFERROR(1-Capacity_Usage!U10/F10,0)</f>
-        <v/>
-      </c>
-      <c r="L10" s="31">
+      <c r="K10" s="32">
+        <f>IF(F10=0,Policy!$B$11,1-Capacity_Usage!U10/F10)</f>
+        <v/>
+      </c>
+      <c r="L10" s="32">
         <f>MIN(MAX(K10,0),1)</f>
         <v/>
       </c>
-      <c r="M10" s="31">
+      <c r="M10" s="32">
         <f>IFERROR(Capacity_Usage!N10/Capacity_Usage!L10,0)</f>
         <v/>
       </c>
-      <c r="N10" s="31">
+      <c r="N10" s="32">
         <f>MIN(MAX(M10,0),1)</f>
         <v/>
       </c>
-      <c r="O10" s="31">
+      <c r="O10" s="32">
         <f>Capacity_Usage!E10/3</f>
         <v/>
       </c>
-      <c r="P10" s="31">
+      <c r="P10" s="32">
         <f>MIN(MAX(O10,0),1)</f>
         <v/>
       </c>
-      <c r="Q10" s="31">
+      <c r="Q10" s="32">
         <f>Policy!$B$2*H10+Policy!$B$3*J10+Policy!$B$4*L10+Policy!$B$5*N10+Policy!$B$6*P10</f>
         <v/>
       </c>
@@ -7455,50 +7416,50 @@
         <v/>
       </c>
       <c r="F11" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C11),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C11,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G11" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C11)</f>
+        <v/>
+      </c>
+      <c r="G11" s="32">
         <f>IFERROR(Capacity_Usage!N11/Capacity_Usage!L11,0)</f>
         <v/>
       </c>
-      <c r="H11" s="31">
+      <c r="H11" s="32">
         <f>MIN(MAX(G11,0),1)</f>
         <v/>
       </c>
-      <c r="I11" s="31">
+      <c r="I11" s="32">
         <f>IFERROR(Capacity_Usage!Q11/Capacity_Usage!O11,0)</f>
         <v/>
       </c>
-      <c r="J11" s="31">
+      <c r="J11" s="32">
         <f>MIN(MAX(I11,0),1)</f>
         <v/>
       </c>
-      <c r="K11" s="31">
-        <f>IFERROR(1-Capacity_Usage!U11/F11,0)</f>
-        <v/>
-      </c>
-      <c r="L11" s="31">
+      <c r="K11" s="32">
+        <f>IF(F11=0,Policy!$B$11,1-Capacity_Usage!U11/F11)</f>
+        <v/>
+      </c>
+      <c r="L11" s="32">
         <f>MIN(MAX(K11,0),1)</f>
         <v/>
       </c>
-      <c r="M11" s="31">
+      <c r="M11" s="32">
         <f>IFERROR(Capacity_Usage!N11/Capacity_Usage!L11,0)</f>
         <v/>
       </c>
-      <c r="N11" s="31">
+      <c r="N11" s="32">
         <f>MIN(MAX(M11,0),1)</f>
         <v/>
       </c>
-      <c r="O11" s="31">
+      <c r="O11" s="32">
         <f>Capacity_Usage!E11/3</f>
         <v/>
       </c>
-      <c r="P11" s="31">
+      <c r="P11" s="32">
         <f>MIN(MAX(O11,0),1)</f>
         <v/>
       </c>
-      <c r="Q11" s="31">
+      <c r="Q11" s="32">
         <f>Policy!$B$2*H11+Policy!$B$3*J11+Policy!$B$4*L11+Policy!$B$5*N11+Policy!$B$6*P11</f>
         <v/>
       </c>
@@ -7533,50 +7494,50 @@
         <v/>
       </c>
       <c r="F12" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C12),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C12,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G12" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C12)</f>
+        <v/>
+      </c>
+      <c r="G12" s="32">
         <f>IFERROR(Capacity_Usage!N12/Capacity_Usage!L12,0)</f>
         <v/>
       </c>
-      <c r="H12" s="31">
+      <c r="H12" s="32">
         <f>MIN(MAX(G12,0),1)</f>
         <v/>
       </c>
-      <c r="I12" s="31">
+      <c r="I12" s="32">
         <f>IFERROR(Capacity_Usage!Q12/Capacity_Usage!O12,0)</f>
         <v/>
       </c>
-      <c r="J12" s="31">
+      <c r="J12" s="32">
         <f>MIN(MAX(I12,0),1)</f>
         <v/>
       </c>
-      <c r="K12" s="31">
-        <f>IFERROR(1-Capacity_Usage!U12/F12,0)</f>
-        <v/>
-      </c>
-      <c r="L12" s="31">
+      <c r="K12" s="32">
+        <f>IF(F12=0,Policy!$B$11,1-Capacity_Usage!U12/F12)</f>
+        <v/>
+      </c>
+      <c r="L12" s="32">
         <f>MIN(MAX(K12,0),1)</f>
         <v/>
       </c>
-      <c r="M12" s="31">
+      <c r="M12" s="32">
         <f>IFERROR(Capacity_Usage!N12/Capacity_Usage!L12,0)</f>
         <v/>
       </c>
-      <c r="N12" s="31">
+      <c r="N12" s="32">
         <f>MIN(MAX(M12,0),1)</f>
         <v/>
       </c>
-      <c r="O12" s="31">
+      <c r="O12" s="32">
         <f>Capacity_Usage!E12/3</f>
         <v/>
       </c>
-      <c r="P12" s="31">
+      <c r="P12" s="32">
         <f>MIN(MAX(O12,0),1)</f>
         <v/>
       </c>
-      <c r="Q12" s="31">
+      <c r="Q12" s="32">
         <f>Policy!$B$2*H12+Policy!$B$3*J12+Policy!$B$4*L12+Policy!$B$5*N12+Policy!$B$6*P12</f>
         <v/>
       </c>
@@ -7611,50 +7572,50 @@
         <v/>
       </c>
       <c r="F13" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C13),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C13,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G13" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C13)</f>
+        <v/>
+      </c>
+      <c r="G13" s="32">
         <f>IFERROR(Capacity_Usage!N13/Capacity_Usage!L13,0)</f>
         <v/>
       </c>
-      <c r="H13" s="31">
+      <c r="H13" s="32">
         <f>MIN(MAX(G13,0),1)</f>
         <v/>
       </c>
-      <c r="I13" s="31">
+      <c r="I13" s="32">
         <f>IFERROR(Capacity_Usage!Q13/Capacity_Usage!O13,0)</f>
         <v/>
       </c>
-      <c r="J13" s="31">
+      <c r="J13" s="32">
         <f>MIN(MAX(I13,0),1)</f>
         <v/>
       </c>
-      <c r="K13" s="31">
-        <f>IFERROR(1-Capacity_Usage!U13/F13,0)</f>
-        <v/>
-      </c>
-      <c r="L13" s="31">
+      <c r="K13" s="32">
+        <f>IF(F13=0,Policy!$B$11,1-Capacity_Usage!U13/F13)</f>
+        <v/>
+      </c>
+      <c r="L13" s="32">
         <f>MIN(MAX(K13,0),1)</f>
         <v/>
       </c>
-      <c r="M13" s="31">
+      <c r="M13" s="32">
         <f>IFERROR(Capacity_Usage!N13/Capacity_Usage!L13,0)</f>
         <v/>
       </c>
-      <c r="N13" s="31">
+      <c r="N13" s="32">
         <f>MIN(MAX(M13,0),1)</f>
         <v/>
       </c>
-      <c r="O13" s="31">
+      <c r="O13" s="32">
         <f>Capacity_Usage!E13/3</f>
         <v/>
       </c>
-      <c r="P13" s="31">
+      <c r="P13" s="32">
         <f>MIN(MAX(O13,0),1)</f>
         <v/>
       </c>
-      <c r="Q13" s="31">
+      <c r="Q13" s="32">
         <f>Policy!$B$2*H13+Policy!$B$3*J13+Policy!$B$4*L13+Policy!$B$5*N13+Policy!$B$6*P13</f>
         <v/>
       </c>
@@ -7689,50 +7650,50 @@
         <v/>
       </c>
       <c r="F14" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C14),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C14,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G14" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C14)</f>
+        <v/>
+      </c>
+      <c r="G14" s="32">
         <f>IFERROR(Capacity_Usage!N14/Capacity_Usage!L14,0)</f>
         <v/>
       </c>
-      <c r="H14" s="31">
+      <c r="H14" s="32">
         <f>MIN(MAX(G14,0),1)</f>
         <v/>
       </c>
-      <c r="I14" s="31">
+      <c r="I14" s="32">
         <f>IFERROR(Capacity_Usage!Q14/Capacity_Usage!O14,0)</f>
         <v/>
       </c>
-      <c r="J14" s="31">
+      <c r="J14" s="32">
         <f>MIN(MAX(I14,0),1)</f>
         <v/>
       </c>
-      <c r="K14" s="31">
-        <f>IFERROR(1-Capacity_Usage!U14/F14,0)</f>
-        <v/>
-      </c>
-      <c r="L14" s="31">
+      <c r="K14" s="32">
+        <f>IF(F14=0,Policy!$B$11,1-Capacity_Usage!U14/F14)</f>
+        <v/>
+      </c>
+      <c r="L14" s="32">
         <f>MIN(MAX(K14,0),1)</f>
         <v/>
       </c>
-      <c r="M14" s="31">
+      <c r="M14" s="32">
         <f>IFERROR(Capacity_Usage!N14/Capacity_Usage!L14,0)</f>
         <v/>
       </c>
-      <c r="N14" s="31">
+      <c r="N14" s="32">
         <f>MIN(MAX(M14,0),1)</f>
         <v/>
       </c>
-      <c r="O14" s="31">
+      <c r="O14" s="32">
         <f>Capacity_Usage!E14/3</f>
         <v/>
       </c>
-      <c r="P14" s="31">
+      <c r="P14" s="32">
         <f>MIN(MAX(O14,0),1)</f>
         <v/>
       </c>
-      <c r="Q14" s="31">
+      <c r="Q14" s="32">
         <f>Policy!$B$2*H14+Policy!$B$3*J14+Policy!$B$4*L14+Policy!$B$5*N14+Policy!$B$6*P14</f>
         <v/>
       </c>
@@ -7767,50 +7728,50 @@
         <v/>
       </c>
       <c r="F15" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C15),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C15,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G15" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C15)</f>
+        <v/>
+      </c>
+      <c r="G15" s="32">
         <f>IFERROR(Capacity_Usage!N15/Capacity_Usage!L15,0)</f>
         <v/>
       </c>
-      <c r="H15" s="31">
+      <c r="H15" s="32">
         <f>MIN(MAX(G15,0),1)</f>
         <v/>
       </c>
-      <c r="I15" s="31">
+      <c r="I15" s="32">
         <f>IFERROR(Capacity_Usage!Q15/Capacity_Usage!O15,0)</f>
         <v/>
       </c>
-      <c r="J15" s="31">
+      <c r="J15" s="32">
         <f>MIN(MAX(I15,0),1)</f>
         <v/>
       </c>
-      <c r="K15" s="31">
-        <f>IFERROR(1-Capacity_Usage!U15/F15,0)</f>
-        <v/>
-      </c>
-      <c r="L15" s="31">
+      <c r="K15" s="32">
+        <f>IF(F15=0,Policy!$B$11,1-Capacity_Usage!U15/F15)</f>
+        <v/>
+      </c>
+      <c r="L15" s="32">
         <f>MIN(MAX(K15,0),1)</f>
         <v/>
       </c>
-      <c r="M15" s="31">
+      <c r="M15" s="32">
         <f>IFERROR(Capacity_Usage!N15/Capacity_Usage!L15,0)</f>
         <v/>
       </c>
-      <c r="N15" s="31">
+      <c r="N15" s="32">
         <f>MIN(MAX(M15,0),1)</f>
         <v/>
       </c>
-      <c r="O15" s="31">
+      <c r="O15" s="32">
         <f>Capacity_Usage!E15/3</f>
         <v/>
       </c>
-      <c r="P15" s="31">
+      <c r="P15" s="32">
         <f>MIN(MAX(O15,0),1)</f>
         <v/>
       </c>
-      <c r="Q15" s="31">
+      <c r="Q15" s="32">
         <f>Policy!$B$2*H15+Policy!$B$3*J15+Policy!$B$4*L15+Policy!$B$5*N15+Policy!$B$6*P15</f>
         <v/>
       </c>
@@ -7845,50 +7806,50 @@
         <v/>
       </c>
       <c r="F16" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C16),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C16,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G16" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C16)</f>
+        <v/>
+      </c>
+      <c r="G16" s="32">
         <f>IFERROR(Capacity_Usage!N16/Capacity_Usage!L16,0)</f>
         <v/>
       </c>
-      <c r="H16" s="31">
+      <c r="H16" s="32">
         <f>MIN(MAX(G16,0),1)</f>
         <v/>
       </c>
-      <c r="I16" s="31">
+      <c r="I16" s="32">
         <f>IFERROR(Capacity_Usage!Q16/Capacity_Usage!O16,0)</f>
         <v/>
       </c>
-      <c r="J16" s="31">
+      <c r="J16" s="32">
         <f>MIN(MAX(I16,0),1)</f>
         <v/>
       </c>
-      <c r="K16" s="31">
-        <f>IFERROR(1-Capacity_Usage!U16/F16,0)</f>
-        <v/>
-      </c>
-      <c r="L16" s="31">
+      <c r="K16" s="32">
+        <f>IF(F16=0,Policy!$B$11,1-Capacity_Usage!U16/F16)</f>
+        <v/>
+      </c>
+      <c r="L16" s="32">
         <f>MIN(MAX(K16,0),1)</f>
         <v/>
       </c>
-      <c r="M16" s="31">
+      <c r="M16" s="32">
         <f>IFERROR(Capacity_Usage!N16/Capacity_Usage!L16,0)</f>
         <v/>
       </c>
-      <c r="N16" s="31">
+      <c r="N16" s="32">
         <f>MIN(MAX(M16,0),1)</f>
         <v/>
       </c>
-      <c r="O16" s="31">
+      <c r="O16" s="32">
         <f>Capacity_Usage!E16/3</f>
         <v/>
       </c>
-      <c r="P16" s="31">
+      <c r="P16" s="32">
         <f>MIN(MAX(O16,0),1)</f>
         <v/>
       </c>
-      <c r="Q16" s="31">
+      <c r="Q16" s="32">
         <f>Policy!$B$2*H16+Policy!$B$3*J16+Policy!$B$4*L16+Policy!$B$5*N16+Policy!$B$6*P16</f>
         <v/>
       </c>
@@ -7923,50 +7884,50 @@
         <v/>
       </c>
       <c r="F17" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C17),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C17,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G17" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C17)</f>
+        <v/>
+      </c>
+      <c r="G17" s="32">
         <f>IFERROR(Capacity_Usage!N17/Capacity_Usage!L17,0)</f>
         <v/>
       </c>
-      <c r="H17" s="31">
+      <c r="H17" s="32">
         <f>MIN(MAX(G17,0),1)</f>
         <v/>
       </c>
-      <c r="I17" s="31">
+      <c r="I17" s="32">
         <f>IFERROR(Capacity_Usage!Q17/Capacity_Usage!O17,0)</f>
         <v/>
       </c>
-      <c r="J17" s="31">
+      <c r="J17" s="32">
         <f>MIN(MAX(I17,0),1)</f>
         <v/>
       </c>
-      <c r="K17" s="31">
-        <f>IFERROR(1-Capacity_Usage!U17/F17,0)</f>
-        <v/>
-      </c>
-      <c r="L17" s="31">
+      <c r="K17" s="32">
+        <f>IF(F17=0,Policy!$B$11,1-Capacity_Usage!U17/F17)</f>
+        <v/>
+      </c>
+      <c r="L17" s="32">
         <f>MIN(MAX(K17,0),1)</f>
         <v/>
       </c>
-      <c r="M17" s="31">
+      <c r="M17" s="32">
         <f>IFERROR(Capacity_Usage!N17/Capacity_Usage!L17,0)</f>
         <v/>
       </c>
-      <c r="N17" s="31">
+      <c r="N17" s="32">
         <f>MIN(MAX(M17,0),1)</f>
         <v/>
       </c>
-      <c r="O17" s="31">
+      <c r="O17" s="32">
         <f>Capacity_Usage!E17/3</f>
         <v/>
       </c>
-      <c r="P17" s="31">
+      <c r="P17" s="32">
         <f>MIN(MAX(O17,0),1)</f>
         <v/>
       </c>
-      <c r="Q17" s="31">
+      <c r="Q17" s="32">
         <f>Policy!$B$2*H17+Policy!$B$3*J17+Policy!$B$4*L17+Policy!$B$5*N17+Policy!$B$6*P17</f>
         <v/>
       </c>
@@ -8022,7 +7983,7 @@
           <t>PS_DR — DR Placement Score  (Middle East scores EU regions cross-geo)</t>
         </is>
       </c>
-      <c r="T1" s="30" t="inlineStr">
+      <c r="T1" s="31" t="inlineStr">
         <is>
           <t>DR WINNER</t>
         </is>
@@ -8140,7 +8101,7 @@
           <t>Score</t>
         </is>
       </c>
-      <c r="U3" s="32">
+      <c r="U3" s="33">
         <f>IF(Setup!$B$10="2-region",Scoring_CVAL!$U$3,IF(MAX(R4:R17)&lt;0,"",MAX(R4:R17)))</f>
         <v/>
       </c>
@@ -8167,50 +8128,50 @@
         <v/>
       </c>
       <c r="F4" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C4),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C4,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G4" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C4)</f>
+        <v/>
+      </c>
+      <c r="G4" s="32">
         <f>IFERROR(Capacity_Usage!S4/Capacity_Usage!R4,0)</f>
         <v/>
       </c>
-      <c r="H4" s="31">
+      <c r="H4" s="32">
         <f>MIN(MAX(G4,0),1)</f>
         <v/>
       </c>
-      <c r="I4" s="31">
+      <c r="I4" s="32">
         <f>IFERROR(Capacity_Usage!Q4/Capacity_Usage!O4,0)</f>
         <v/>
       </c>
-      <c r="J4" s="31">
+      <c r="J4" s="32">
         <f>MIN(MAX(I4,0),1)</f>
         <v/>
       </c>
-      <c r="K4" s="31">
-        <f>IFERROR(1-Capacity_Usage!U4/F4,0)</f>
-        <v/>
-      </c>
-      <c r="L4" s="31">
+      <c r="K4" s="32">
+        <f>IF(F4=0,Policy!$B$11,1-Capacity_Usage!U4/F4)</f>
+        <v/>
+      </c>
+      <c r="L4" s="32">
         <f>MIN(MAX(K4,0),1)</f>
         <v/>
       </c>
-      <c r="M4" s="31">
+      <c r="M4" s="32">
         <f>IFERROR(Capacity_Usage!T4/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N4" s="31">
+      <c r="N4" s="32">
         <f>MIN(MAX(M4,0),1)</f>
         <v/>
       </c>
-      <c r="O4" s="31">
+      <c r="O4" s="32">
         <f>Capacity_Usage!E4/3</f>
         <v/>
       </c>
-      <c r="P4" s="31">
+      <c r="P4" s="32">
         <f>MIN(MAX(O4,0),1)</f>
         <v/>
       </c>
-      <c r="Q4" s="31">
+      <c r="Q4" s="32">
         <f>Policy!$B$2*H4+Policy!$B$3*J4+Policy!$B$4*L4+Policy!$B$5*N4+Policy!$B$6*P4</f>
         <v/>
       </c>
@@ -8245,50 +8206,50 @@
         <v/>
       </c>
       <c r="F5" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C5),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C5,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G5" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C5)</f>
+        <v/>
+      </c>
+      <c r="G5" s="32">
         <f>IFERROR(Capacity_Usage!S5/Capacity_Usage!R5,0)</f>
         <v/>
       </c>
-      <c r="H5" s="31">
+      <c r="H5" s="32">
         <f>MIN(MAX(G5,0),1)</f>
         <v/>
       </c>
-      <c r="I5" s="31">
+      <c r="I5" s="32">
         <f>IFERROR(Capacity_Usage!Q5/Capacity_Usage!O5,0)</f>
         <v/>
       </c>
-      <c r="J5" s="31">
+      <c r="J5" s="32">
         <f>MIN(MAX(I5,0),1)</f>
         <v/>
       </c>
-      <c r="K5" s="31">
-        <f>IFERROR(1-Capacity_Usage!U5/F5,0)</f>
-        <v/>
-      </c>
-      <c r="L5" s="31">
+      <c r="K5" s="32">
+        <f>IF(F5=0,Policy!$B$11,1-Capacity_Usage!U5/F5)</f>
+        <v/>
+      </c>
+      <c r="L5" s="32">
         <f>MIN(MAX(K5,0),1)</f>
         <v/>
       </c>
-      <c r="M5" s="31">
+      <c r="M5" s="32">
         <f>IFERROR(Capacity_Usage!T5/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N5" s="31">
+      <c r="N5" s="32">
         <f>MIN(MAX(M5,0),1)</f>
         <v/>
       </c>
-      <c r="O5" s="31">
+      <c r="O5" s="32">
         <f>Capacity_Usage!E5/3</f>
         <v/>
       </c>
-      <c r="P5" s="31">
+      <c r="P5" s="32">
         <f>MIN(MAX(O5,0),1)</f>
         <v/>
       </c>
-      <c r="Q5" s="31">
+      <c r="Q5" s="32">
         <f>Policy!$B$2*H5+Policy!$B$3*J5+Policy!$B$4*L5+Policy!$B$5*N5+Policy!$B$6*P5</f>
         <v/>
       </c>
@@ -8323,50 +8284,50 @@
         <v/>
       </c>
       <c r="F6" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C6),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C6,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G6" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C6)</f>
+        <v/>
+      </c>
+      <c r="G6" s="32">
         <f>IFERROR(Capacity_Usage!S6/Capacity_Usage!R6,0)</f>
         <v/>
       </c>
-      <c r="H6" s="31">
+      <c r="H6" s="32">
         <f>MIN(MAX(G6,0),1)</f>
         <v/>
       </c>
-      <c r="I6" s="31">
+      <c r="I6" s="32">
         <f>IFERROR(Capacity_Usage!Q6/Capacity_Usage!O6,0)</f>
         <v/>
       </c>
-      <c r="J6" s="31">
+      <c r="J6" s="32">
         <f>MIN(MAX(I6,0),1)</f>
         <v/>
       </c>
-      <c r="K6" s="31">
-        <f>IFERROR(1-Capacity_Usage!U6/F6,0)</f>
-        <v/>
-      </c>
-      <c r="L6" s="31">
+      <c r="K6" s="32">
+        <f>IF(F6=0,Policy!$B$11,1-Capacity_Usage!U6/F6)</f>
+        <v/>
+      </c>
+      <c r="L6" s="32">
         <f>MIN(MAX(K6,0),1)</f>
         <v/>
       </c>
-      <c r="M6" s="31">
+      <c r="M6" s="32">
         <f>IFERROR(Capacity_Usage!T6/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N6" s="31">
+      <c r="N6" s="32">
         <f>MIN(MAX(M6,0),1)</f>
         <v/>
       </c>
-      <c r="O6" s="31">
+      <c r="O6" s="32">
         <f>Capacity_Usage!E6/3</f>
         <v/>
       </c>
-      <c r="P6" s="31">
+      <c r="P6" s="32">
         <f>MIN(MAX(O6,0),1)</f>
         <v/>
       </c>
-      <c r="Q6" s="31">
+      <c r="Q6" s="32">
         <f>Policy!$B$2*H6+Policy!$B$3*J6+Policy!$B$4*L6+Policy!$B$5*N6+Policy!$B$6*P6</f>
         <v/>
       </c>
@@ -8401,50 +8362,50 @@
         <v/>
       </c>
       <c r="F7" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C7),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C7,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G7" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C7)</f>
+        <v/>
+      </c>
+      <c r="G7" s="32">
         <f>IFERROR(Capacity_Usage!S7/Capacity_Usage!R7,0)</f>
         <v/>
       </c>
-      <c r="H7" s="31">
+      <c r="H7" s="32">
         <f>MIN(MAX(G7,0),1)</f>
         <v/>
       </c>
-      <c r="I7" s="31">
+      <c r="I7" s="32">
         <f>IFERROR(Capacity_Usage!Q7/Capacity_Usage!O7,0)</f>
         <v/>
       </c>
-      <c r="J7" s="31">
+      <c r="J7" s="32">
         <f>MIN(MAX(I7,0),1)</f>
         <v/>
       </c>
-      <c r="K7" s="31">
-        <f>IFERROR(1-Capacity_Usage!U7/F7,0)</f>
-        <v/>
-      </c>
-      <c r="L7" s="31">
+      <c r="K7" s="32">
+        <f>IF(F7=0,Policy!$B$11,1-Capacity_Usage!U7/F7)</f>
+        <v/>
+      </c>
+      <c r="L7" s="32">
         <f>MIN(MAX(K7,0),1)</f>
         <v/>
       </c>
-      <c r="M7" s="31">
+      <c r="M7" s="32">
         <f>IFERROR(Capacity_Usage!T7/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N7" s="31">
+      <c r="N7" s="32">
         <f>MIN(MAX(M7,0),1)</f>
         <v/>
       </c>
-      <c r="O7" s="31">
+      <c r="O7" s="32">
         <f>Capacity_Usage!E7/3</f>
         <v/>
       </c>
-      <c r="P7" s="31">
+      <c r="P7" s="32">
         <f>MIN(MAX(O7,0),1)</f>
         <v/>
       </c>
-      <c r="Q7" s="31">
+      <c r="Q7" s="32">
         <f>Policy!$B$2*H7+Policy!$B$3*J7+Policy!$B$4*L7+Policy!$B$5*N7+Policy!$B$6*P7</f>
         <v/>
       </c>
@@ -8479,50 +8440,50 @@
         <v/>
       </c>
       <c r="F8" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C8),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C8,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G8" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C8)</f>
+        <v/>
+      </c>
+      <c r="G8" s="32">
         <f>IFERROR(Capacity_Usage!S8/Capacity_Usage!R8,0)</f>
         <v/>
       </c>
-      <c r="H8" s="31">
+      <c r="H8" s="32">
         <f>MIN(MAX(G8,0),1)</f>
         <v/>
       </c>
-      <c r="I8" s="31">
+      <c r="I8" s="32">
         <f>IFERROR(Capacity_Usage!Q8/Capacity_Usage!O8,0)</f>
         <v/>
       </c>
-      <c r="J8" s="31">
+      <c r="J8" s="32">
         <f>MIN(MAX(I8,0),1)</f>
         <v/>
       </c>
-      <c r="K8" s="31">
-        <f>IFERROR(1-Capacity_Usage!U8/F8,0)</f>
-        <v/>
-      </c>
-      <c r="L8" s="31">
+      <c r="K8" s="32">
+        <f>IF(F8=0,Policy!$B$11,1-Capacity_Usage!U8/F8)</f>
+        <v/>
+      </c>
+      <c r="L8" s="32">
         <f>MIN(MAX(K8,0),1)</f>
         <v/>
       </c>
-      <c r="M8" s="31">
+      <c r="M8" s="32">
         <f>IFERROR(Capacity_Usage!T8/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N8" s="31">
+      <c r="N8" s="32">
         <f>MIN(MAX(M8,0),1)</f>
         <v/>
       </c>
-      <c r="O8" s="31">
+      <c r="O8" s="32">
         <f>Capacity_Usage!E8/3</f>
         <v/>
       </c>
-      <c r="P8" s="31">
+      <c r="P8" s="32">
         <f>MIN(MAX(O8,0),1)</f>
         <v/>
       </c>
-      <c r="Q8" s="31">
+      <c r="Q8" s="32">
         <f>Policy!$B$2*H8+Policy!$B$3*J8+Policy!$B$4*L8+Policy!$B$5*N8+Policy!$B$6*P8</f>
         <v/>
       </c>
@@ -8557,50 +8518,50 @@
         <v/>
       </c>
       <c r="F9" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C9),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C9,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G9" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C9)</f>
+        <v/>
+      </c>
+      <c r="G9" s="32">
         <f>IFERROR(Capacity_Usage!S9/Capacity_Usage!R9,0)</f>
         <v/>
       </c>
-      <c r="H9" s="31">
+      <c r="H9" s="32">
         <f>MIN(MAX(G9,0),1)</f>
         <v/>
       </c>
-      <c r="I9" s="31">
+      <c r="I9" s="32">
         <f>IFERROR(Capacity_Usage!Q9/Capacity_Usage!O9,0)</f>
         <v/>
       </c>
-      <c r="J9" s="31">
+      <c r="J9" s="32">
         <f>MIN(MAX(I9,0),1)</f>
         <v/>
       </c>
-      <c r="K9" s="31">
-        <f>IFERROR(1-Capacity_Usage!U9/F9,0)</f>
-        <v/>
-      </c>
-      <c r="L9" s="31">
+      <c r="K9" s="32">
+        <f>IF(F9=0,Policy!$B$11,1-Capacity_Usage!U9/F9)</f>
+        <v/>
+      </c>
+      <c r="L9" s="32">
         <f>MIN(MAX(K9,0),1)</f>
         <v/>
       </c>
-      <c r="M9" s="31">
+      <c r="M9" s="32">
         <f>IFERROR(Capacity_Usage!T9/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N9" s="31">
+      <c r="N9" s="32">
         <f>MIN(MAX(M9,0),1)</f>
         <v/>
       </c>
-      <c r="O9" s="31">
+      <c r="O9" s="32">
         <f>Capacity_Usage!E9/3</f>
         <v/>
       </c>
-      <c r="P9" s="31">
+      <c r="P9" s="32">
         <f>MIN(MAX(O9,0),1)</f>
         <v/>
       </c>
-      <c r="Q9" s="31">
+      <c r="Q9" s="32">
         <f>Policy!$B$2*H9+Policy!$B$3*J9+Policy!$B$4*L9+Policy!$B$5*N9+Policy!$B$6*P9</f>
         <v/>
       </c>
@@ -8635,50 +8596,50 @@
         <v/>
       </c>
       <c r="F10" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C10),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C10,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G10" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C10)</f>
+        <v/>
+      </c>
+      <c r="G10" s="32">
         <f>IFERROR(Capacity_Usage!S10/Capacity_Usage!R10,0)</f>
         <v/>
       </c>
-      <c r="H10" s="31">
+      <c r="H10" s="32">
         <f>MIN(MAX(G10,0),1)</f>
         <v/>
       </c>
-      <c r="I10" s="31">
+      <c r="I10" s="32">
         <f>IFERROR(Capacity_Usage!Q10/Capacity_Usage!O10,0)</f>
         <v/>
       </c>
-      <c r="J10" s="31">
+      <c r="J10" s="32">
         <f>MIN(MAX(I10,0),1)</f>
         <v/>
       </c>
-      <c r="K10" s="31">
-        <f>IFERROR(1-Capacity_Usage!U10/F10,0)</f>
-        <v/>
-      </c>
-      <c r="L10" s="31">
+      <c r="K10" s="32">
+        <f>IF(F10=0,Policy!$B$11,1-Capacity_Usage!U10/F10)</f>
+        <v/>
+      </c>
+      <c r="L10" s="32">
         <f>MIN(MAX(K10,0),1)</f>
         <v/>
       </c>
-      <c r="M10" s="31">
+      <c r="M10" s="32">
         <f>IFERROR(Capacity_Usage!T10/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N10" s="31">
+      <c r="N10" s="32">
         <f>MIN(MAX(M10,0),1)</f>
         <v/>
       </c>
-      <c r="O10" s="31">
+      <c r="O10" s="32">
         <f>Capacity_Usage!E10/3</f>
         <v/>
       </c>
-      <c r="P10" s="31">
+      <c r="P10" s="32">
         <f>MIN(MAX(O10,0),1)</f>
         <v/>
       </c>
-      <c r="Q10" s="31">
+      <c r="Q10" s="32">
         <f>Policy!$B$2*H10+Policy!$B$3*J10+Policy!$B$4*L10+Policy!$B$5*N10+Policy!$B$6*P10</f>
         <v/>
       </c>
@@ -8713,50 +8674,50 @@
         <v/>
       </c>
       <c r="F11" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C11),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C11,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G11" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C11)</f>
+        <v/>
+      </c>
+      <c r="G11" s="32">
         <f>IFERROR(Capacity_Usage!S11/Capacity_Usage!R11,0)</f>
         <v/>
       </c>
-      <c r="H11" s="31">
+      <c r="H11" s="32">
         <f>MIN(MAX(G11,0),1)</f>
         <v/>
       </c>
-      <c r="I11" s="31">
+      <c r="I11" s="32">
         <f>IFERROR(Capacity_Usage!Q11/Capacity_Usage!O11,0)</f>
         <v/>
       </c>
-      <c r="J11" s="31">
+      <c r="J11" s="32">
         <f>MIN(MAX(I11,0),1)</f>
         <v/>
       </c>
-      <c r="K11" s="31">
-        <f>IFERROR(1-Capacity_Usage!U11/F11,0)</f>
-        <v/>
-      </c>
-      <c r="L11" s="31">
+      <c r="K11" s="32">
+        <f>IF(F11=0,Policy!$B$11,1-Capacity_Usage!U11/F11)</f>
+        <v/>
+      </c>
+      <c r="L11" s="32">
         <f>MIN(MAX(K11,0),1)</f>
         <v/>
       </c>
-      <c r="M11" s="31">
+      <c r="M11" s="32">
         <f>IFERROR(Capacity_Usage!T11/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N11" s="31">
+      <c r="N11" s="32">
         <f>MIN(MAX(M11,0),1)</f>
         <v/>
       </c>
-      <c r="O11" s="31">
+      <c r="O11" s="32">
         <f>Capacity_Usage!E11/3</f>
         <v/>
       </c>
-      <c r="P11" s="31">
+      <c r="P11" s="32">
         <f>MIN(MAX(O11,0),1)</f>
         <v/>
       </c>
-      <c r="Q11" s="31">
+      <c r="Q11" s="32">
         <f>Policy!$B$2*H11+Policy!$B$3*J11+Policy!$B$4*L11+Policy!$B$5*N11+Policy!$B$6*P11</f>
         <v/>
       </c>
@@ -8791,50 +8752,50 @@
         <v/>
       </c>
       <c r="F12" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C12),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C12,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G12" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C12)</f>
+        <v/>
+      </c>
+      <c r="G12" s="32">
         <f>IFERROR(Capacity_Usage!S12/Capacity_Usage!R12,0)</f>
         <v/>
       </c>
-      <c r="H12" s="31">
+      <c r="H12" s="32">
         <f>MIN(MAX(G12,0),1)</f>
         <v/>
       </c>
-      <c r="I12" s="31">
+      <c r="I12" s="32">
         <f>IFERROR(Capacity_Usage!Q12/Capacity_Usage!O12,0)</f>
         <v/>
       </c>
-      <c r="J12" s="31">
+      <c r="J12" s="32">
         <f>MIN(MAX(I12,0),1)</f>
         <v/>
       </c>
-      <c r="K12" s="31">
-        <f>IFERROR(1-Capacity_Usage!U12/F12,0)</f>
-        <v/>
-      </c>
-      <c r="L12" s="31">
+      <c r="K12" s="32">
+        <f>IF(F12=0,Policy!$B$11,1-Capacity_Usage!U12/F12)</f>
+        <v/>
+      </c>
+      <c r="L12" s="32">
         <f>MIN(MAX(K12,0),1)</f>
         <v/>
       </c>
-      <c r="M12" s="31">
+      <c r="M12" s="32">
         <f>IFERROR(Capacity_Usage!T12/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N12" s="31">
+      <c r="N12" s="32">
         <f>MIN(MAX(M12,0),1)</f>
         <v/>
       </c>
-      <c r="O12" s="31">
+      <c r="O12" s="32">
         <f>Capacity_Usage!E12/3</f>
         <v/>
       </c>
-      <c r="P12" s="31">
+      <c r="P12" s="32">
         <f>MIN(MAX(O12,0),1)</f>
         <v/>
       </c>
-      <c r="Q12" s="31">
+      <c r="Q12" s="32">
         <f>Policy!$B$2*H12+Policy!$B$3*J12+Policy!$B$4*L12+Policy!$B$5*N12+Policy!$B$6*P12</f>
         <v/>
       </c>
@@ -8869,50 +8830,50 @@
         <v/>
       </c>
       <c r="F13" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C13),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C13,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G13" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C13)</f>
+        <v/>
+      </c>
+      <c r="G13" s="32">
         <f>IFERROR(Capacity_Usage!S13/Capacity_Usage!R13,0)</f>
         <v/>
       </c>
-      <c r="H13" s="31">
+      <c r="H13" s="32">
         <f>MIN(MAX(G13,0),1)</f>
         <v/>
       </c>
-      <c r="I13" s="31">
+      <c r="I13" s="32">
         <f>IFERROR(Capacity_Usage!Q13/Capacity_Usage!O13,0)</f>
         <v/>
       </c>
-      <c r="J13" s="31">
+      <c r="J13" s="32">
         <f>MIN(MAX(I13,0),1)</f>
         <v/>
       </c>
-      <c r="K13" s="31">
-        <f>IFERROR(1-Capacity_Usage!U13/F13,0)</f>
-        <v/>
-      </c>
-      <c r="L13" s="31">
+      <c r="K13" s="32">
+        <f>IF(F13=0,Policy!$B$11,1-Capacity_Usage!U13/F13)</f>
+        <v/>
+      </c>
+      <c r="L13" s="32">
         <f>MIN(MAX(K13,0),1)</f>
         <v/>
       </c>
-      <c r="M13" s="31">
+      <c r="M13" s="32">
         <f>IFERROR(Capacity_Usage!T13/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N13" s="31">
+      <c r="N13" s="32">
         <f>MIN(MAX(M13,0),1)</f>
         <v/>
       </c>
-      <c r="O13" s="31">
+      <c r="O13" s="32">
         <f>Capacity_Usage!E13/3</f>
         <v/>
       </c>
-      <c r="P13" s="31">
+      <c r="P13" s="32">
         <f>MIN(MAX(O13,0),1)</f>
         <v/>
       </c>
-      <c r="Q13" s="31">
+      <c r="Q13" s="32">
         <f>Policy!$B$2*H13+Policy!$B$3*J13+Policy!$B$4*L13+Policy!$B$5*N13+Policy!$B$6*P13</f>
         <v/>
       </c>
@@ -8947,50 +8908,50 @@
         <v/>
       </c>
       <c r="F14" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C14),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C14,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G14" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C14)</f>
+        <v/>
+      </c>
+      <c r="G14" s="32">
         <f>IFERROR(Capacity_Usage!S14/Capacity_Usage!R14,0)</f>
         <v/>
       </c>
-      <c r="H14" s="31">
+      <c r="H14" s="32">
         <f>MIN(MAX(G14,0),1)</f>
         <v/>
       </c>
-      <c r="I14" s="31">
+      <c r="I14" s="32">
         <f>IFERROR(Capacity_Usage!Q14/Capacity_Usage!O14,0)</f>
         <v/>
       </c>
-      <c r="J14" s="31">
+      <c r="J14" s="32">
         <f>MIN(MAX(I14,0),1)</f>
         <v/>
       </c>
-      <c r="K14" s="31">
-        <f>IFERROR(1-Capacity_Usage!U14/F14,0)</f>
-        <v/>
-      </c>
-      <c r="L14" s="31">
+      <c r="K14" s="32">
+        <f>IF(F14=0,Policy!$B$11,1-Capacity_Usage!U14/F14)</f>
+        <v/>
+      </c>
+      <c r="L14" s="32">
         <f>MIN(MAX(K14,0),1)</f>
         <v/>
       </c>
-      <c r="M14" s="31">
+      <c r="M14" s="32">
         <f>IFERROR(Capacity_Usage!T14/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N14" s="31">
+      <c r="N14" s="32">
         <f>MIN(MAX(M14,0),1)</f>
         <v/>
       </c>
-      <c r="O14" s="31">
+      <c r="O14" s="32">
         <f>Capacity_Usage!E14/3</f>
         <v/>
       </c>
-      <c r="P14" s="31">
+      <c r="P14" s="32">
         <f>MIN(MAX(O14,0),1)</f>
         <v/>
       </c>
-      <c r="Q14" s="31">
+      <c r="Q14" s="32">
         <f>Policy!$B$2*H14+Policy!$B$3*J14+Policy!$B$4*L14+Policy!$B$5*N14+Policy!$B$6*P14</f>
         <v/>
       </c>
@@ -9025,50 +8986,50 @@
         <v/>
       </c>
       <c r="F15" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C15),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C15,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G15" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C15)</f>
+        <v/>
+      </c>
+      <c r="G15" s="32">
         <f>IFERROR(Capacity_Usage!S15/Capacity_Usage!R15,0)</f>
         <v/>
       </c>
-      <c r="H15" s="31">
+      <c r="H15" s="32">
         <f>MIN(MAX(G15,0),1)</f>
         <v/>
       </c>
-      <c r="I15" s="31">
+      <c r="I15" s="32">
         <f>IFERROR(Capacity_Usage!Q15/Capacity_Usage!O15,0)</f>
         <v/>
       </c>
-      <c r="J15" s="31">
+      <c r="J15" s="32">
         <f>MIN(MAX(I15,0),1)</f>
         <v/>
       </c>
-      <c r="K15" s="31">
-        <f>IFERROR(1-Capacity_Usage!U15/F15,0)</f>
-        <v/>
-      </c>
-      <c r="L15" s="31">
+      <c r="K15" s="32">
+        <f>IF(F15=0,Policy!$B$11,1-Capacity_Usage!U15/F15)</f>
+        <v/>
+      </c>
+      <c r="L15" s="32">
         <f>MIN(MAX(K15,0),1)</f>
         <v/>
       </c>
-      <c r="M15" s="31">
+      <c r="M15" s="32">
         <f>IFERROR(Capacity_Usage!T15/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N15" s="31">
+      <c r="N15" s="32">
         <f>MIN(MAX(M15,0),1)</f>
         <v/>
       </c>
-      <c r="O15" s="31">
+      <c r="O15" s="32">
         <f>Capacity_Usage!E15/3</f>
         <v/>
       </c>
-      <c r="P15" s="31">
+      <c r="P15" s="32">
         <f>MIN(MAX(O15,0),1)</f>
         <v/>
       </c>
-      <c r="Q15" s="31">
+      <c r="Q15" s="32">
         <f>Policy!$B$2*H15+Policy!$B$3*J15+Policy!$B$4*L15+Policy!$B$5*N15+Policy!$B$6*P15</f>
         <v/>
       </c>
@@ -9103,50 +9064,50 @@
         <v/>
       </c>
       <c r="F16" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C16),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C16,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G16" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C16)</f>
+        <v/>
+      </c>
+      <c r="G16" s="32">
         <f>IFERROR(Capacity_Usage!S16/Capacity_Usage!R16,0)</f>
         <v/>
       </c>
-      <c r="H16" s="31">
+      <c r="H16" s="32">
         <f>MIN(MAX(G16,0),1)</f>
         <v/>
       </c>
-      <c r="I16" s="31">
+      <c r="I16" s="32">
         <f>IFERROR(Capacity_Usage!Q16/Capacity_Usage!O16,0)</f>
         <v/>
       </c>
-      <c r="J16" s="31">
+      <c r="J16" s="32">
         <f>MIN(MAX(I16,0),1)</f>
         <v/>
       </c>
-      <c r="K16" s="31">
-        <f>IFERROR(1-Capacity_Usage!U16/F16,0)</f>
-        <v/>
-      </c>
-      <c r="L16" s="31">
+      <c r="K16" s="32">
+        <f>IF(F16=0,Policy!$B$11,1-Capacity_Usage!U16/F16)</f>
+        <v/>
+      </c>
+      <c r="L16" s="32">
         <f>MIN(MAX(K16,0),1)</f>
         <v/>
       </c>
-      <c r="M16" s="31">
+      <c r="M16" s="32">
         <f>IFERROR(Capacity_Usage!T16/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N16" s="31">
+      <c r="N16" s="32">
         <f>MIN(MAX(M16,0),1)</f>
         <v/>
       </c>
-      <c r="O16" s="31">
+      <c r="O16" s="32">
         <f>Capacity_Usage!E16/3</f>
         <v/>
       </c>
-      <c r="P16" s="31">
+      <c r="P16" s="32">
         <f>MIN(MAX(O16,0),1)</f>
         <v/>
       </c>
-      <c r="Q16" s="31">
+      <c r="Q16" s="32">
         <f>Policy!$B$2*H16+Policy!$B$3*J16+Policy!$B$4*L16+Policy!$B$5*N16+Policy!$B$6*P16</f>
         <v/>
       </c>
@@ -9181,50 +9142,50 @@
         <v/>
       </c>
       <c r="F17" s="12">
-        <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C17),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C17,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
-        <v/>
-      </c>
-      <c r="G17" s="31">
+        <f>SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C17)</f>
+        <v/>
+      </c>
+      <c r="G17" s="32">
         <f>IFERROR(Capacity_Usage!S17/Capacity_Usage!R17,0)</f>
         <v/>
       </c>
-      <c r="H17" s="31">
+      <c r="H17" s="32">
         <f>MIN(MAX(G17,0),1)</f>
         <v/>
       </c>
-      <c r="I17" s="31">
+      <c r="I17" s="32">
         <f>IFERROR(Capacity_Usage!Q17/Capacity_Usage!O17,0)</f>
         <v/>
       </c>
-      <c r="J17" s="31">
+      <c r="J17" s="32">
         <f>MIN(MAX(I17,0),1)</f>
         <v/>
       </c>
-      <c r="K17" s="31">
-        <f>IFERROR(1-Capacity_Usage!U17/F17,0)</f>
-        <v/>
-      </c>
-      <c r="L17" s="31">
+      <c r="K17" s="32">
+        <f>IF(F17=0,Policy!$B$11,1-Capacity_Usage!U17/F17)</f>
+        <v/>
+      </c>
+      <c r="L17" s="32">
         <f>MIN(MAX(K17,0),1)</f>
         <v/>
       </c>
-      <c r="M17" s="31">
+      <c r="M17" s="32">
         <f>IFERROR(Capacity_Usage!T17/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N17" s="31">
+      <c r="N17" s="32">
         <f>MIN(MAX(M17,0),1)</f>
         <v/>
       </c>
-      <c r="O17" s="31">
+      <c r="O17" s="32">
         <f>Capacity_Usage!E17/3</f>
         <v/>
       </c>
-      <c r="P17" s="31">
+      <c r="P17" s="32">
         <f>MIN(MAX(O17,0),1)</f>
         <v/>
       </c>
-      <c r="Q17" s="31">
+      <c r="Q17" s="32">
         <f>Policy!$B$2*H17+Policy!$B$3*J17+Policy!$B$4*L17+Policy!$B$5*N17+Policy!$B$6*P17</f>
         <v/>
       </c>

</xml_diff>